<commit_message>
NBFC flow part1+part2 brd for nbfc implementation as well as agreement permanant initate
</commit_message>
<xml_diff>
--- a/Itarang_Work_Report_3_Months_2026-05-25.xlsx
+++ b/Itarang_Work_Report_3_Months_2026-05-25.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EF0A7C-6BBD-44C8-922E-EC84C0A33045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55859C38-C20D-44B0-B831-FE0972B1A015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,13 +15,14 @@
     <sheet name="NBFC Onboarding" sheetId="5" r:id="rId5"/>
     <sheet name="NBFC Dashboard" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2587" uniqueCount="1298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2628" uniqueCount="1301">
   <si>
     <t>iTarang — 3-Month Work Report</t>
   </si>
@@ -3915,6 +3916,15 @@
   </si>
   <si>
     <t>Testing pending</t>
+  </si>
+  <si>
+    <t>5.  NBFC Addendum (V1 +V2)</t>
+  </si>
+  <si>
+    <t>LIST OF CHANGES</t>
+  </si>
+  <si>
+    <t>ZOHO Integration</t>
   </si>
 </sst>
 </file>
@@ -3999,7 +4009,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4070,6 +4080,12 @@
         <fgColor rgb="FF404040"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -4131,7 +4147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4164,6 +4180,15 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -4176,34 +4201,34 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4214,21 +4239,15 @@
     <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4581,36 +4600,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
     </row>
     <row r="8" spans="1:5" ht="22.05" customHeight="1">
       <c r="A8" s="1" t="s">
@@ -4697,13 +4716,21 @@
         <v>1297</v>
       </c>
     </row>
+    <row r="13" spans="1:5">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1300</v>
+      </c>
+    </row>
     <row r="15" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
     </row>
     <row r="16" spans="1:5" ht="27.6">
       <c r="A16" s="5" t="s">
@@ -4796,34 +4823,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
@@ -4938,12 +4965,12 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
@@ -4960,23 +4987,23 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
       <c r="E18" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
@@ -5049,12 +5076,12 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
     </row>
     <row r="27" spans="1:5" ht="27.6">
       <c r="A27" s="5" t="s">
@@ -5085,23 +5112,23 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
       <c r="E31" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
     </row>
     <row r="33" spans="1:4" ht="27.6">
       <c r="A33" s="5" t="s">
@@ -5160,12 +5187,12 @@
       </c>
     </row>
     <row r="38" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
@@ -5196,12 +5223,12 @@
       </c>
     </row>
     <row r="42" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="5" t="s">
@@ -5246,12 +5273,12 @@
       </c>
     </row>
     <row r="47" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A47" s="17" t="s">
+      <c r="A47" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="5" t="s">
@@ -5296,23 +5323,23 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A53" s="19" t="s">
+      <c r="A53" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="B53" s="19"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="21"/>
       <c r="E53" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A54" s="17" t="s">
+      <c r="A54" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
@@ -5343,12 +5370,12 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A58" s="17" t="s">
+      <c r="A58" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="17"/>
+      <c r="B58" s="20"/>
+      <c r="C58" s="20"/>
+      <c r="D58" s="20"/>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="5" t="s">
@@ -5407,23 +5434,23 @@
       </c>
     </row>
     <row r="65" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A65" s="19" t="s">
+      <c r="A65" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="B65" s="19"/>
-      <c r="C65" s="19"/>
-      <c r="D65" s="19"/>
+      <c r="B65" s="21"/>
+      <c r="C65" s="21"/>
+      <c r="D65" s="21"/>
       <c r="E65" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A66" s="17" t="s">
+      <c r="A66" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="5" t="s">
@@ -5454,12 +5481,12 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A70" s="17" t="s">
+      <c r="A70" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17"/>
+      <c r="B70" s="20"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="20"/>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="5" t="s">
@@ -5504,12 +5531,12 @@
       </c>
     </row>
     <row r="75" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A75" s="17" t="s">
+      <c r="A75" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="B75" s="17"/>
-      <c r="C75" s="17"/>
-      <c r="D75" s="17"/>
+      <c r="B75" s="20"/>
+      <c r="C75" s="20"/>
+      <c r="D75" s="20"/>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" s="5" t="s">
@@ -5526,12 +5553,12 @@
       </c>
     </row>
     <row r="78" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A78" s="17" t="s">
+      <c r="A78" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="B78" s="17"/>
-      <c r="C78" s="17"/>
-      <c r="D78" s="17"/>
+      <c r="B78" s="20"/>
+      <c r="C78" s="20"/>
+      <c r="D78" s="20"/>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="5" t="s">
@@ -5562,12 +5589,12 @@
       </c>
     </row>
     <row r="82" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="B82" s="17"/>
-      <c r="C82" s="17"/>
-      <c r="D82" s="17"/>
+      <c r="B82" s="20"/>
+      <c r="C82" s="20"/>
+      <c r="D82" s="20"/>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="5" t="s">
@@ -5612,12 +5639,12 @@
       </c>
     </row>
     <row r="87" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A87" s="17" t="s">
+      <c r="A87" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="B87" s="17"/>
-      <c r="C87" s="17"/>
-      <c r="D87" s="17"/>
+      <c r="B87" s="20"/>
+      <c r="C87" s="20"/>
+      <c r="D87" s="20"/>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" s="5" t="s">
@@ -5634,23 +5661,23 @@
       </c>
     </row>
     <row r="91" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A91" s="19" t="s">
+      <c r="A91" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B91" s="19"/>
-      <c r="C91" s="19"/>
-      <c r="D91" s="19"/>
+      <c r="B91" s="21"/>
+      <c r="C91" s="21"/>
+      <c r="D91" s="21"/>
       <c r="E91" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A92" s="17" t="s">
+      <c r="A92" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="B92" s="17"/>
-      <c r="C92" s="17"/>
-      <c r="D92" s="17"/>
+      <c r="B92" s="20"/>
+      <c r="C92" s="20"/>
+      <c r="D92" s="20"/>
     </row>
     <row r="93" spans="1:5">
       <c r="A93" s="5" t="s">
@@ -5807,12 +5834,12 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A105" s="17" t="s">
+      <c r="A105" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="B105" s="17"/>
-      <c r="C105" s="17"/>
-      <c r="D105" s="17"/>
+      <c r="B105" s="20"/>
+      <c r="C105" s="20"/>
+      <c r="D105" s="20"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="5" t="s">
@@ -5857,12 +5884,12 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A110" s="17" t="s">
+      <c r="A110" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="B110" s="17"/>
-      <c r="C110" s="17"/>
-      <c r="D110" s="17"/>
+      <c r="B110" s="20"/>
+      <c r="C110" s="20"/>
+      <c r="D110" s="20"/>
     </row>
     <row r="111" spans="1:4" ht="27.6">
       <c r="A111" s="5" t="s">
@@ -5936,32 +5963,32 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="A78:D78"/>
     <mergeCell ref="A110:D110"/>
     <mergeCell ref="A82:D82"/>
     <mergeCell ref="A87:D87"/>
     <mergeCell ref="A91:D91"/>
     <mergeCell ref="A92:D92"/>
     <mergeCell ref="A105:D105"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A18:D18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -5983,34 +6010,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
       <c r="E4" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6030,12 +6057,12 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6083,12 +6110,12 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
       <c r="E12" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6122,23 +6149,23 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="23" t="s">
         <v>204</v>
       </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
       <c r="E17" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6214,12 +6241,12 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
       <c r="E25" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6337,12 +6364,12 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="20" t="s">
         <v>233</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
       <c r="E35" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6432,12 +6459,12 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="20" t="s">
         <v>246</v>
       </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
       <c r="E43" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6569,12 +6596,12 @@
       </c>
     </row>
     <row r="54" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A54" s="17" t="s">
+      <c r="A54" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
       <c r="E54" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6622,12 +6649,12 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A59" s="17" t="s">
+      <c r="A59" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
+      <c r="B59" s="20"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="20"/>
       <c r="E59" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6773,12 +6800,12 @@
       </c>
     </row>
     <row r="71" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A71" s="17" t="s">
+      <c r="A71" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="B71" s="17"/>
-      <c r="C71" s="17"/>
-      <c r="D71" s="17"/>
+      <c r="B71" s="20"/>
+      <c r="C71" s="20"/>
+      <c r="D71" s="20"/>
       <c r="E71" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6924,12 +6951,12 @@
       </c>
     </row>
     <row r="83" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A83" s="17" t="s">
+      <c r="A83" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="B83" s="17"/>
-      <c r="C83" s="17"/>
-      <c r="D83" s="17"/>
+      <c r="B83" s="20"/>
+      <c r="C83" s="20"/>
+      <c r="D83" s="20"/>
       <c r="E83" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6949,12 +6976,12 @@
       </c>
     </row>
     <row r="86" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A86" s="17" t="s">
+      <c r="A86" s="20" t="s">
         <v>317</v>
       </c>
-      <c r="B86" s="17"/>
-      <c r="C86" s="17"/>
-      <c r="D86" s="17"/>
+      <c r="B86" s="20"/>
+      <c r="C86" s="20"/>
+      <c r="D86" s="20"/>
       <c r="E86" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7044,12 +7071,12 @@
       </c>
     </row>
     <row r="94" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A94" s="17" t="s">
+      <c r="A94" s="20" t="s">
         <v>331</v>
       </c>
-      <c r="B94" s="17"/>
-      <c r="C94" s="17"/>
-      <c r="D94" s="17"/>
+      <c r="B94" s="20"/>
+      <c r="C94" s="20"/>
+      <c r="D94" s="20"/>
       <c r="E94" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7125,12 +7152,12 @@
       </c>
     </row>
     <row r="101" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A101" s="17" t="s">
+      <c r="A101" s="20" t="s">
         <v>342</v>
       </c>
-      <c r="B101" s="17"/>
-      <c r="C101" s="17"/>
-      <c r="D101" s="17"/>
+      <c r="B101" s="20"/>
+      <c r="C101" s="20"/>
+      <c r="D101" s="20"/>
       <c r="E101" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7248,12 +7275,12 @@
       </c>
     </row>
     <row r="111" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A111" s="17" t="s">
+      <c r="A111" s="20" t="s">
         <v>361</v>
       </c>
-      <c r="B111" s="17"/>
-      <c r="C111" s="17"/>
-      <c r="D111" s="17"/>
+      <c r="B111" s="20"/>
+      <c r="C111" s="20"/>
+      <c r="D111" s="20"/>
       <c r="E111" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7469,23 +7496,23 @@
       </c>
     </row>
     <row r="129" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A129" s="21" t="s">
+      <c r="A129" s="23" t="s">
         <v>392</v>
       </c>
-      <c r="B129" s="21"/>
-      <c r="C129" s="21"/>
-      <c r="D129" s="21"/>
+      <c r="B129" s="23"/>
+      <c r="C129" s="23"/>
+      <c r="D129" s="23"/>
       <c r="E129" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="130" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A130" s="17" t="s">
+      <c r="A130" s="20" t="s">
         <v>393</v>
       </c>
-      <c r="B130" s="17"/>
-      <c r="C130" s="17"/>
-      <c r="D130" s="17"/>
+      <c r="B130" s="20"/>
+      <c r="C130" s="20"/>
+      <c r="D130" s="20"/>
     </row>
     <row r="131" spans="1:5" ht="27.6">
       <c r="A131" s="5" t="s">
@@ -7810,12 +7837,12 @@
       </c>
     </row>
     <row r="155" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A155" s="17" t="s">
+      <c r="A155" s="20" t="s">
         <v>440</v>
       </c>
-      <c r="B155" s="17"/>
-      <c r="C155" s="17"/>
-      <c r="D155" s="17"/>
+      <c r="B155" s="20"/>
+      <c r="C155" s="20"/>
+      <c r="D155" s="20"/>
       <c r="E155" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7891,12 +7918,12 @@
       </c>
     </row>
     <row r="162" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A162" s="17" t="s">
+      <c r="A162" s="20" t="s">
         <v>451</v>
       </c>
-      <c r="B162" s="17"/>
-      <c r="C162" s="17"/>
-      <c r="D162" s="17"/>
+      <c r="B162" s="20"/>
+      <c r="C162" s="20"/>
+      <c r="D162" s="20"/>
       <c r="E162" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7930,12 +7957,12 @@
       </c>
     </row>
     <row r="166" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A166" s="17" t="s">
+      <c r="A166" s="20" t="s">
         <v>456</v>
       </c>
-      <c r="B166" s="17"/>
-      <c r="C166" s="17"/>
-      <c r="D166" s="17"/>
+      <c r="B166" s="20"/>
+      <c r="C166" s="20"/>
+      <c r="D166" s="20"/>
       <c r="E166" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7969,12 +7996,12 @@
       </c>
     </row>
     <row r="170" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A170" s="17" t="s">
+      <c r="A170" s="20" t="s">
         <v>459</v>
       </c>
-      <c r="B170" s="17"/>
-      <c r="C170" s="17"/>
-      <c r="D170" s="17"/>
+      <c r="B170" s="20"/>
+      <c r="C170" s="20"/>
+      <c r="D170" s="20"/>
       <c r="E170" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8008,12 +8035,12 @@
       </c>
     </row>
     <row r="174" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A174" s="17" t="s">
+      <c r="A174" s="20" t="s">
         <v>462</v>
       </c>
-      <c r="B174" s="17"/>
-      <c r="C174" s="17"/>
-      <c r="D174" s="17"/>
+      <c r="B174" s="20"/>
+      <c r="C174" s="20"/>
+      <c r="D174" s="20"/>
       <c r="E174" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8089,12 +8116,12 @@
       </c>
     </row>
     <row r="181" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A181" s="17" t="s">
+      <c r="A181" s="20" t="s">
         <v>473</v>
       </c>
-      <c r="B181" s="17"/>
-      <c r="C181" s="17"/>
-      <c r="D181" s="17"/>
+      <c r="B181" s="20"/>
+      <c r="C181" s="20"/>
+      <c r="D181" s="20"/>
       <c r="E181" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8156,12 +8183,12 @@
       </c>
     </row>
     <row r="187" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A187" s="17" t="s">
+      <c r="A187" s="20" t="s">
         <v>482</v>
       </c>
-      <c r="B187" s="17"/>
-      <c r="C187" s="17"/>
-      <c r="D187" s="17"/>
+      <c r="B187" s="20"/>
+      <c r="C187" s="20"/>
+      <c r="D187" s="20"/>
       <c r="E187" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8237,12 +8264,12 @@
       </c>
     </row>
     <row r="194" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A194" s="17" t="s">
+      <c r="A194" s="20" t="s">
         <v>492</v>
       </c>
-      <c r="B194" s="17"/>
-      <c r="C194" s="17"/>
-      <c r="D194" s="17"/>
+      <c r="B194" s="20"/>
+      <c r="C194" s="20"/>
+      <c r="D194" s="20"/>
       <c r="E194" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8347,6 +8374,26 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A71:D71"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A111:D111"/>
+    <mergeCell ref="A129:D129"/>
+    <mergeCell ref="A130:D130"/>
     <mergeCell ref="A181:D181"/>
     <mergeCell ref="A187:D187"/>
     <mergeCell ref="A194:D194"/>
@@ -8355,26 +8402,6 @@
     <mergeCell ref="A166:D166"/>
     <mergeCell ref="A170:D170"/>
     <mergeCell ref="A174:D174"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A111:D111"/>
-    <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A130:D130"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A86:D86"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A12:D12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -8396,34 +8423,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="26" t="s">
         <v>506</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="25" t="s">
         <v>507</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>508</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
     </row>
     <row r="5" spans="1:5" ht="27.6">
       <c r="A5" s="5" t="s">
@@ -8496,12 +8523,12 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="20" t="s">
         <v>519</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
       <c r="E11" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8577,12 +8604,12 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="20" t="s">
         <v>528</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
       <c r="E18" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8896,12 +8923,12 @@
       </c>
     </row>
     <row r="42" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A42" s="17" t="s">
+      <c r="A42" s="20" t="s">
         <v>573</v>
       </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
+      <c r="B42" s="20"/>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
       <c r="E42" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9033,12 +9060,12 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A53" s="17" t="s">
+      <c r="A53" s="20" t="s">
         <v>590</v>
       </c>
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
+      <c r="B53" s="20"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="20"/>
       <c r="E53" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9198,12 +9225,12 @@
       </c>
     </row>
     <row r="66" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A66" s="17" t="s">
+      <c r="A66" s="20" t="s">
         <v>613</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
       <c r="E66" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9279,12 +9306,12 @@
       </c>
     </row>
     <row r="73" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A73" s="17" t="s">
+      <c r="A73" s="20" t="s">
         <v>624</v>
       </c>
-      <c r="B73" s="17"/>
-      <c r="C73" s="17"/>
-      <c r="D73" s="17"/>
+      <c r="B73" s="20"/>
+      <c r="C73" s="20"/>
+      <c r="D73" s="20"/>
       <c r="E73" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9388,12 +9415,12 @@
       </c>
     </row>
     <row r="82" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A82" s="17" t="s">
+      <c r="A82" s="20" t="s">
         <v>639</v>
       </c>
-      <c r="B82" s="17"/>
-      <c r="C82" s="17"/>
-      <c r="D82" s="17"/>
+      <c r="B82" s="20"/>
+      <c r="C82" s="20"/>
+      <c r="D82" s="20"/>
       <c r="E82" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9497,12 +9524,12 @@
       </c>
     </row>
     <row r="91" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A91" s="17" t="s">
+      <c r="A91" s="20" t="s">
         <v>654</v>
       </c>
-      <c r="B91" s="17"/>
-      <c r="C91" s="17"/>
-      <c r="D91" s="17"/>
+      <c r="B91" s="20"/>
+      <c r="C91" s="20"/>
+      <c r="D91" s="20"/>
       <c r="E91" s="11" t="s">
         <v>1273</v>
       </c>
@@ -9577,7 +9604,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="52.8">
+    <row r="97" spans="1:5" ht="66">
       <c r="A97" s="5" t="s">
         <v>25</v>
       </c>
@@ -9732,12 +9759,12 @@
       </c>
     </row>
     <row r="109" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A109" s="17" t="s">
+      <c r="A109" s="20" t="s">
         <v>687</v>
       </c>
-      <c r="B109" s="17"/>
-      <c r="C109" s="17"/>
-      <c r="D109" s="17"/>
+      <c r="B109" s="20"/>
+      <c r="C109" s="20"/>
+      <c r="D109" s="20"/>
       <c r="E109" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9813,12 +9840,12 @@
       </c>
     </row>
     <row r="116" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A116" s="17" t="s">
+      <c r="A116" s="20" t="s">
         <v>696</v>
       </c>
-      <c r="B116" s="17"/>
-      <c r="C116" s="17"/>
-      <c r="D116" s="17"/>
+      <c r="B116" s="20"/>
+      <c r="C116" s="20"/>
+      <c r="D116" s="20"/>
       <c r="E116" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9922,23 +9949,23 @@
       </c>
     </row>
     <row r="126" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A126" s="23" t="s">
+      <c r="A126" s="25" t="s">
         <v>708</v>
       </c>
-      <c r="B126" s="23"/>
-      <c r="C126" s="23"/>
-      <c r="D126" s="23"/>
+      <c r="B126" s="25"/>
+      <c r="C126" s="25"/>
+      <c r="D126" s="25"/>
       <c r="E126" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="128" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A128" s="17" t="s">
+      <c r="A128" s="20" t="s">
         <v>709</v>
       </c>
-      <c r="B128" s="17"/>
-      <c r="C128" s="17"/>
-      <c r="D128" s="17"/>
+      <c r="B128" s="20"/>
+      <c r="C128" s="20"/>
+      <c r="D128" s="20"/>
     </row>
     <row r="129" spans="1:4" ht="27.6">
       <c r="A129" s="5" t="s">
@@ -9972,21 +9999,21 @@
     <row r="136" spans="1:4" ht="19.95" customHeight="1"/>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A73:D73"/>
+    <mergeCell ref="A82:D82"/>
     <mergeCell ref="A128:D128"/>
     <mergeCell ref="A91:D91"/>
     <mergeCell ref="A109:D109"/>
     <mergeCell ref="A116:D116"/>
     <mergeCell ref="A126:D126"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A73:D73"/>
-    <mergeCell ref="A82:D82"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A18:D18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -10008,34 +10035,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="28" t="s">
         <v>714</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="27" t="s">
         <v>715</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>716</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
@@ -10108,12 +10135,12 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="20" t="s">
         <v>726</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
@@ -10144,12 +10171,12 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="20" t="s">
         <v>731</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="5" t="s">
@@ -10166,12 +10193,12 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="20" t="s">
         <v>734</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="5" t="s">
@@ -10230,12 +10257,12 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="20" t="s">
         <v>743</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="5" t="s">
@@ -10280,12 +10307,12 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="20" t="s">
         <v>749</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
@@ -10330,23 +10357,23 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A35" s="25" t="s">
+      <c r="A35" s="27" t="s">
         <v>756</v>
       </c>
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
       <c r="E35" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="20" t="s">
         <v>757</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="5" t="s">
@@ -10475,12 +10502,12 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A47" s="17" t="s">
+      <c r="A47" s="20" t="s">
         <v>768</v>
       </c>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="5" t="s">
@@ -10525,23 +10552,23 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A53" s="25" t="s">
+      <c r="A53" s="27" t="s">
         <v>775</v>
       </c>
-      <c r="B53" s="25"/>
-      <c r="C53" s="25"/>
-      <c r="D53" s="25"/>
+      <c r="B53" s="27"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="27"/>
       <c r="E53" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A54" s="17" t="s">
+      <c r="A54" s="20" t="s">
         <v>776</v>
       </c>
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
@@ -10586,12 +10613,12 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A59" s="17" t="s">
+      <c r="A59" s="20" t="s">
         <v>783</v>
       </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
+      <c r="B59" s="20"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="20"/>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="5" t="s">
@@ -10636,12 +10663,12 @@
       </c>
     </row>
     <row r="64" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A64" s="17" t="s">
+      <c r="A64" s="20" t="s">
         <v>788</v>
       </c>
-      <c r="B64" s="17"/>
-      <c r="C64" s="17"/>
-      <c r="D64" s="17"/>
+      <c r="B64" s="20"/>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="5" t="s">
@@ -10686,23 +10713,23 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A70" s="25" t="s">
+      <c r="A70" s="27" t="s">
         <v>794</v>
       </c>
-      <c r="B70" s="25"/>
-      <c r="C70" s="25"/>
-      <c r="D70" s="25"/>
+      <c r="B70" s="27"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="27"/>
       <c r="E70" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A71" s="17" t="s">
+      <c r="A71" s="20" t="s">
         <v>795</v>
       </c>
-      <c r="B71" s="17"/>
-      <c r="C71" s="17"/>
-      <c r="D71" s="17"/>
+      <c r="B71" s="20"/>
+      <c r="C71" s="20"/>
+      <c r="D71" s="20"/>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="5" t="s">
@@ -10775,12 +10802,12 @@
       </c>
     </row>
     <row r="78" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A78" s="17" t="s">
+      <c r="A78" s="20" t="s">
         <v>806</v>
       </c>
-      <c r="B78" s="17"/>
-      <c r="C78" s="17"/>
-      <c r="D78" s="17"/>
+      <c r="B78" s="20"/>
+      <c r="C78" s="20"/>
+      <c r="D78" s="20"/>
     </row>
     <row r="79" spans="1:5" ht="27.6">
       <c r="A79" s="5" t="s">
@@ -10797,12 +10824,12 @@
       </c>
     </row>
     <row r="81" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A81" s="17" t="s">
+      <c r="A81" s="20" t="s">
         <v>809</v>
       </c>
-      <c r="B81" s="17"/>
-      <c r="C81" s="17"/>
-      <c r="D81" s="17"/>
+      <c r="B81" s="20"/>
+      <c r="C81" s="20"/>
+      <c r="D81" s="20"/>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="5" t="s">
@@ -10847,23 +10874,23 @@
       </c>
     </row>
     <row r="87" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A87" s="25" t="s">
+      <c r="A87" s="27" t="s">
         <v>816</v>
       </c>
-      <c r="B87" s="25"/>
-      <c r="C87" s="25"/>
-      <c r="D87" s="25"/>
+      <c r="B87" s="27"/>
+      <c r="C87" s="27"/>
+      <c r="D87" s="27"/>
       <c r="E87" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A88" s="17" t="s">
+      <c r="A88" s="20" t="s">
         <v>817</v>
       </c>
-      <c r="B88" s="17"/>
-      <c r="C88" s="17"/>
-      <c r="D88" s="17"/>
+      <c r="B88" s="20"/>
+      <c r="C88" s="20"/>
+      <c r="D88" s="20"/>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" s="5" t="s">
@@ -10908,12 +10935,12 @@
       </c>
     </row>
     <row r="93" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A93" s="17" t="s">
+      <c r="A93" s="20" t="s">
         <v>823</v>
       </c>
-      <c r="B93" s="17"/>
-      <c r="C93" s="17"/>
-      <c r="D93" s="17"/>
+      <c r="B93" s="20"/>
+      <c r="C93" s="20"/>
+      <c r="D93" s="20"/>
     </row>
     <row r="94" spans="1:5">
       <c r="A94" s="5" t="s">
@@ -10945,6 +10972,21 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A53:D53"/>
+    <mergeCell ref="A54:D54"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A64:D64"/>
     <mergeCell ref="A88:D88"/>
     <mergeCell ref="A93:D93"/>
     <mergeCell ref="A70:D70"/>
@@ -10952,21 +10994,6 @@
     <mergeCell ref="A78:D78"/>
     <mergeCell ref="A81:D81"/>
     <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -10988,34 +11015,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="30" t="s">
         <v>828</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="29" t="s">
         <v>829</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
       <c r="E3" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>830</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
@@ -11074,12 +11101,12 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="20" t="s">
         <v>839</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
@@ -11152,12 +11179,12 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="20" t="s">
         <v>850</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
     </row>
     <row r="18" spans="1:5" ht="39.6">
       <c r="A18" s="5" t="s">
@@ -11188,12 +11215,12 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
     </row>
     <row r="22" spans="1:5" ht="55.2">
       <c r="A22" s="5" t="s">
@@ -11224,12 +11251,12 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
     </row>
     <row r="26" spans="1:5" ht="27.6">
       <c r="A26" s="5" t="s">
@@ -11246,23 +11273,23 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="29" t="s">
         <v>865</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
       <c r="E29" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="20" t="s">
         <v>866</v>
       </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="5" t="s">
@@ -11419,12 +11446,12 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="20" t="s">
         <v>888</v>
       </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
     </row>
     <row r="44" spans="1:4" ht="27.6">
       <c r="A44" s="5" t="s">
@@ -11497,12 +11524,12 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A50" s="17" t="s">
+      <c r="A50" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B50" s="17"/>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
     </row>
     <row r="51" spans="1:5" ht="41.4">
       <c r="A51" s="5" t="s">
@@ -11547,12 +11574,12 @@
       </c>
     </row>
     <row r="55" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A55" s="17" t="s">
+      <c r="A55" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
-      <c r="D55" s="17"/>
+      <c r="B55" s="20"/>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="5" t="s">
@@ -11583,23 +11610,23 @@
       </c>
     </row>
     <row r="60" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A60" s="27" t="s">
+      <c r="A60" s="29" t="s">
         <v>909</v>
       </c>
-      <c r="B60" s="27"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="27"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="29"/>
+      <c r="D60" s="29"/>
       <c r="E60" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A61" s="17" t="s">
+      <c r="A61" s="20" t="s">
         <v>910</v>
       </c>
-      <c r="B61" s="17"/>
-      <c r="C61" s="17"/>
-      <c r="D61" s="17"/>
+      <c r="B61" s="20"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="5" t="s">
@@ -11658,12 +11685,12 @@
       </c>
     </row>
     <row r="67" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A67" s="17" t="s">
+      <c r="A67" s="20" t="s">
         <v>919</v>
       </c>
-      <c r="B67" s="17"/>
-      <c r="C67" s="17"/>
-      <c r="D67" s="17"/>
+      <c r="B67" s="20"/>
+      <c r="C67" s="20"/>
+      <c r="D67" s="20"/>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="5" t="s">
@@ -11736,12 +11763,12 @@
       </c>
     </row>
     <row r="74" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A74" s="17" t="s">
+      <c r="A74" s="20" t="s">
         <v>891</v>
       </c>
-      <c r="B74" s="17"/>
-      <c r="C74" s="17"/>
-      <c r="D74" s="17"/>
+      <c r="B74" s="20"/>
+      <c r="C74" s="20"/>
+      <c r="D74" s="20"/>
     </row>
     <row r="75" spans="1:4" ht="26.4">
       <c r="A75" s="5" t="s">
@@ -11842,12 +11869,12 @@
       </c>
     </row>
     <row r="83" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A83" s="17" t="s">
+      <c r="A83" s="20" t="s">
         <v>943</v>
       </c>
-      <c r="B83" s="17"/>
-      <c r="C83" s="17"/>
-      <c r="D83" s="17"/>
+      <c r="B83" s="20"/>
+      <c r="C83" s="20"/>
+      <c r="D83" s="20"/>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="5" t="s">
@@ -11934,12 +11961,12 @@
       </c>
     </row>
     <row r="91" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A91" s="17" t="s">
+      <c r="A91" s="20" t="s">
         <v>956</v>
       </c>
-      <c r="B91" s="17"/>
-      <c r="C91" s="17"/>
-      <c r="D91" s="17"/>
+      <c r="B91" s="20"/>
+      <c r="C91" s="20"/>
+      <c r="D91" s="20"/>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="5" t="s">
@@ -11998,12 +12025,12 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A97" s="17" t="s">
+      <c r="A97" s="20" t="s">
         <v>964</v>
       </c>
-      <c r="B97" s="17"/>
-      <c r="C97" s="17"/>
-      <c r="D97" s="17"/>
+      <c r="B97" s="20"/>
+      <c r="C97" s="20"/>
+      <c r="D97" s="20"/>
     </row>
     <row r="98" spans="1:4" ht="27.6">
       <c r="A98" s="5" t="s">
@@ -12020,12 +12047,12 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A100" s="17" t="s">
+      <c r="A100" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B100" s="17"/>
-      <c r="C100" s="17"/>
-      <c r="D100" s="17"/>
+      <c r="B100" s="20"/>
+      <c r="C100" s="20"/>
+      <c r="D100" s="20"/>
     </row>
     <row r="101" spans="1:4" ht="96.6">
       <c r="A101" s="5" t="s">
@@ -12070,12 +12097,12 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A105" s="17" t="s">
+      <c r="A105" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B105" s="17"/>
-      <c r="C105" s="17"/>
-      <c r="D105" s="17"/>
+      <c r="B105" s="20"/>
+      <c r="C105" s="20"/>
+      <c r="D105" s="20"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="5" t="s">
@@ -12148,23 +12175,23 @@
       </c>
     </row>
     <row r="113" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A113" s="27" t="s">
+      <c r="A113" s="29" t="s">
         <v>983</v>
       </c>
-      <c r="B113" s="27"/>
-      <c r="C113" s="27"/>
-      <c r="D113" s="27"/>
+      <c r="B113" s="29"/>
+      <c r="C113" s="29"/>
+      <c r="D113" s="29"/>
       <c r="E113" s="11" t="s">
         <v>1273</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A114" s="17" t="s">
+      <c r="A114" s="20" t="s">
         <v>984</v>
       </c>
-      <c r="B114" s="17"/>
-      <c r="C114" s="17"/>
-      <c r="D114" s="17"/>
+      <c r="B114" s="20"/>
+      <c r="C114" s="20"/>
+      <c r="D114" s="20"/>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" s="5" t="s">
@@ -12223,12 +12250,12 @@
       </c>
     </row>
     <row r="120" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A120" s="17" t="s">
+      <c r="A120" s="20" t="s">
         <v>993</v>
       </c>
-      <c r="B120" s="17"/>
-      <c r="C120" s="17"/>
-      <c r="D120" s="17"/>
+      <c r="B120" s="20"/>
+      <c r="C120" s="20"/>
+      <c r="D120" s="20"/>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" s="5" t="s">
@@ -12315,12 +12342,12 @@
       </c>
     </row>
     <row r="128" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A128" s="17" t="s">
+      <c r="A128" s="20" t="s">
         <v>1006</v>
       </c>
-      <c r="B128" s="17"/>
-      <c r="C128" s="17"/>
-      <c r="D128" s="17"/>
+      <c r="B128" s="20"/>
+      <c r="C128" s="20"/>
+      <c r="D128" s="20"/>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="5" t="s">
@@ -12351,12 +12378,12 @@
       </c>
     </row>
     <row r="132" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A132" s="17" t="s">
+      <c r="A132" s="20" t="s">
         <v>1011</v>
       </c>
-      <c r="B132" s="17"/>
-      <c r="C132" s="17"/>
-      <c r="D132" s="17"/>
+      <c r="B132" s="20"/>
+      <c r="C132" s="20"/>
+      <c r="D132" s="20"/>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="5" t="s">
@@ -12429,12 +12456,12 @@
       </c>
     </row>
     <row r="139" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A139" s="17" t="s">
+      <c r="A139" s="20" t="s">
         <v>1019</v>
       </c>
-      <c r="B139" s="17"/>
-      <c r="C139" s="17"/>
-      <c r="D139" s="17"/>
+      <c r="B139" s="20"/>
+      <c r="C139" s="20"/>
+      <c r="D139" s="20"/>
     </row>
     <row r="140" spans="1:4" ht="39.6">
       <c r="A140" s="5" t="s">
@@ -12465,12 +12492,12 @@
       </c>
     </row>
     <row r="143" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A143" s="17" t="s">
+      <c r="A143" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B143" s="17"/>
-      <c r="C143" s="17"/>
-      <c r="D143" s="17"/>
+      <c r="B143" s="20"/>
+      <c r="C143" s="20"/>
+      <c r="D143" s="20"/>
     </row>
     <row r="144" spans="1:4" ht="69">
       <c r="A144" s="5" t="s">
@@ -12515,12 +12542,12 @@
       </c>
     </row>
     <row r="148" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A148" s="17" t="s">
+      <c r="A148" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B148" s="17"/>
-      <c r="C148" s="17"/>
-      <c r="D148" s="17"/>
+      <c r="B148" s="20"/>
+      <c r="C148" s="20"/>
+      <c r="D148" s="20"/>
     </row>
     <row r="149" spans="1:5">
       <c r="A149" s="5" t="s">
@@ -12551,23 +12578,23 @@
       </c>
     </row>
     <row r="153" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A153" s="27" t="s">
+      <c r="A153" s="29" t="s">
         <v>1033</v>
       </c>
-      <c r="B153" s="27"/>
-      <c r="C153" s="27"/>
-      <c r="D153" s="27"/>
+      <c r="B153" s="29"/>
+      <c r="C153" s="29"/>
+      <c r="D153" s="29"/>
       <c r="E153" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="154" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A154" s="17" t="s">
+      <c r="A154" s="20" t="s">
         <v>1034</v>
       </c>
-      <c r="B154" s="17"/>
-      <c r="C154" s="17"/>
-      <c r="D154" s="17"/>
+      <c r="B154" s="20"/>
+      <c r="C154" s="20"/>
+      <c r="D154" s="20"/>
     </row>
     <row r="155" spans="1:5" ht="26.4">
       <c r="A155" s="5" t="s">
@@ -12626,12 +12653,12 @@
       </c>
     </row>
     <row r="160" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A160" s="17" t="s">
+      <c r="A160" s="20" t="s">
         <v>1043</v>
       </c>
-      <c r="B160" s="17"/>
-      <c r="C160" s="17"/>
-      <c r="D160" s="17"/>
+      <c r="B160" s="20"/>
+      <c r="C160" s="20"/>
+      <c r="D160" s="20"/>
     </row>
     <row r="161" spans="1:4" ht="27.6">
       <c r="A161" s="5" t="s">
@@ -12690,12 +12717,12 @@
       </c>
     </row>
     <row r="166" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A166" s="17" t="s">
+      <c r="A166" s="20" t="s">
         <v>1052</v>
       </c>
-      <c r="B166" s="17"/>
-      <c r="C166" s="17"/>
-      <c r="D166" s="17"/>
+      <c r="B166" s="20"/>
+      <c r="C166" s="20"/>
+      <c r="D166" s="20"/>
     </row>
     <row r="167" spans="1:4" ht="26.4">
       <c r="A167" s="5" t="s">
@@ -12740,12 +12767,12 @@
       </c>
     </row>
     <row r="171" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A171" s="17" t="s">
+      <c r="A171" s="20" t="s">
         <v>1058</v>
       </c>
-      <c r="B171" s="17"/>
-      <c r="C171" s="17"/>
-      <c r="D171" s="17"/>
+      <c r="B171" s="20"/>
+      <c r="C171" s="20"/>
+      <c r="D171" s="20"/>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="5" t="s">
@@ -12776,12 +12803,12 @@
       </c>
     </row>
     <row r="175" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A175" s="17" t="s">
+      <c r="A175" s="20" t="s">
         <v>1063</v>
       </c>
-      <c r="B175" s="17"/>
-      <c r="C175" s="17"/>
-      <c r="D175" s="17"/>
+      <c r="B175" s="20"/>
+      <c r="C175" s="20"/>
+      <c r="D175" s="20"/>
     </row>
     <row r="176" spans="1:4" ht="27.6">
       <c r="A176" s="5" t="s">
@@ -12798,12 +12825,12 @@
       </c>
     </row>
     <row r="178" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A178" s="17" t="s">
+      <c r="A178" s="20" t="s">
         <v>1066</v>
       </c>
-      <c r="B178" s="17"/>
-      <c r="C178" s="17"/>
-      <c r="D178" s="17"/>
+      <c r="B178" s="20"/>
+      <c r="C178" s="20"/>
+      <c r="D178" s="20"/>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" s="5" t="s">
@@ -12862,12 +12889,12 @@
       </c>
     </row>
     <row r="184" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A184" s="17" t="s">
+      <c r="A184" s="20" t="s">
         <v>1075</v>
       </c>
-      <c r="B184" s="17"/>
-      <c r="C184" s="17"/>
-      <c r="D184" s="17"/>
+      <c r="B184" s="20"/>
+      <c r="C184" s="20"/>
+      <c r="D184" s="20"/>
     </row>
     <row r="185" spans="1:4">
       <c r="A185" s="5" t="s">
@@ -12912,12 +12939,12 @@
       </c>
     </row>
     <row r="189" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A189" s="17" t="s">
+      <c r="A189" s="20" t="s">
         <v>1081</v>
       </c>
-      <c r="B189" s="17"/>
-      <c r="C189" s="17"/>
-      <c r="D189" s="17"/>
+      <c r="B189" s="20"/>
+      <c r="C189" s="20"/>
+      <c r="D189" s="20"/>
     </row>
     <row r="190" spans="1:4" ht="39.6">
       <c r="A190" s="5" t="s">
@@ -12976,12 +13003,12 @@
       </c>
     </row>
     <row r="195" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A195" s="17" t="s">
+      <c r="A195" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B195" s="17"/>
-      <c r="C195" s="17"/>
-      <c r="D195" s="17"/>
+      <c r="B195" s="20"/>
+      <c r="C195" s="20"/>
+      <c r="D195" s="20"/>
     </row>
     <row r="196" spans="1:4" ht="55.2">
       <c r="A196" s="5" t="s">
@@ -13054,12 +13081,12 @@
       </c>
     </row>
     <row r="202" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A202" s="17" t="s">
+      <c r="A202" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B202" s="17"/>
-      <c r="C202" s="17"/>
-      <c r="D202" s="17"/>
+      <c r="B202" s="20"/>
+      <c r="C202" s="20"/>
+      <c r="D202" s="20"/>
     </row>
     <row r="203" spans="1:4">
       <c r="A203" s="5" t="s">
@@ -13146,23 +13173,23 @@
       </c>
     </row>
     <row r="211" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A211" s="27" t="s">
+      <c r="A211" s="29" t="s">
         <v>1111</v>
       </c>
-      <c r="B211" s="27"/>
-      <c r="C211" s="27"/>
-      <c r="D211" s="27"/>
+      <c r="B211" s="29"/>
+      <c r="C211" s="29"/>
+      <c r="D211" s="29"/>
       <c r="E211" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="212" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A212" s="17" t="s">
+      <c r="A212" s="20" t="s">
         <v>1112</v>
       </c>
-      <c r="B212" s="17"/>
-      <c r="C212" s="17"/>
-      <c r="D212" s="17"/>
+      <c r="B212" s="20"/>
+      <c r="C212" s="20"/>
+      <c r="D212" s="20"/>
     </row>
     <row r="213" spans="1:5">
       <c r="A213" s="5" t="s">
@@ -13235,12 +13262,12 @@
       </c>
     </row>
     <row r="219" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A219" s="17" t="s">
+      <c r="A219" s="20" t="s">
         <v>1122</v>
       </c>
-      <c r="B219" s="17"/>
-      <c r="C219" s="17"/>
-      <c r="D219" s="17"/>
+      <c r="B219" s="20"/>
+      <c r="C219" s="20"/>
+      <c r="D219" s="20"/>
     </row>
     <row r="220" spans="1:5" ht="27.6">
       <c r="A220" s="5" t="s">
@@ -13271,12 +13298,12 @@
       </c>
     </row>
     <row r="223" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A223" s="17" t="s">
+      <c r="A223" s="20" t="s">
         <v>1125</v>
       </c>
-      <c r="B223" s="17"/>
-      <c r="C223" s="17"/>
-      <c r="D223" s="17"/>
+      <c r="B223" s="20"/>
+      <c r="C223" s="20"/>
+      <c r="D223" s="20"/>
     </row>
     <row r="224" spans="1:5">
       <c r="A224" s="5" t="s">
@@ -13307,12 +13334,12 @@
       </c>
     </row>
     <row r="227" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A227" s="17" t="s">
+      <c r="A227" s="20" t="s">
         <v>850</v>
       </c>
-      <c r="B227" s="17"/>
-      <c r="C227" s="17"/>
-      <c r="D227" s="17"/>
+      <c r="B227" s="20"/>
+      <c r="C227" s="20"/>
+      <c r="D227" s="20"/>
     </row>
     <row r="228" spans="1:4">
       <c r="A228" s="5" t="s">
@@ -13357,12 +13384,12 @@
       </c>
     </row>
     <row r="232" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A232" s="17" t="s">
+      <c r="A232" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B232" s="17"/>
-      <c r="C232" s="17"/>
-      <c r="D232" s="17"/>
+      <c r="B232" s="20"/>
+      <c r="C232" s="20"/>
+      <c r="D232" s="20"/>
     </row>
     <row r="233" spans="1:4" ht="55.2">
       <c r="A233" s="5" t="s">
@@ -13421,12 +13448,12 @@
       </c>
     </row>
     <row r="238" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A238" s="17" t="s">
+      <c r="A238" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B238" s="17"/>
-      <c r="C238" s="17"/>
-      <c r="D238" s="17"/>
+      <c r="B238" s="20"/>
+      <c r="C238" s="20"/>
+      <c r="D238" s="20"/>
     </row>
     <row r="239" spans="1:4">
       <c r="A239" s="5" t="s">
@@ -13471,23 +13498,23 @@
       </c>
     </row>
     <row r="244" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A244" s="27" t="s">
+      <c r="A244" s="29" t="s">
         <v>1147</v>
       </c>
-      <c r="B244" s="27"/>
-      <c r="C244" s="27"/>
-      <c r="D244" s="27"/>
+      <c r="B244" s="29"/>
+      <c r="C244" s="29"/>
+      <c r="D244" s="29"/>
       <c r="E244" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="245" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A245" s="17" t="s">
+      <c r="A245" s="20" t="s">
         <v>1148</v>
       </c>
-      <c r="B245" s="17"/>
-      <c r="C245" s="17"/>
-      <c r="D245" s="17"/>
+      <c r="B245" s="20"/>
+      <c r="C245" s="20"/>
+      <c r="D245" s="20"/>
     </row>
     <row r="246" spans="1:5">
       <c r="A246" s="5" t="s">
@@ -13504,12 +13531,12 @@
       </c>
     </row>
     <row r="248" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A248" s="17" t="s">
+      <c r="A248" s="20" t="s">
         <v>1151</v>
       </c>
-      <c r="B248" s="17"/>
-      <c r="C248" s="17"/>
-      <c r="D248" s="17"/>
+      <c r="B248" s="20"/>
+      <c r="C248" s="20"/>
+      <c r="D248" s="20"/>
     </row>
     <row r="249" spans="1:5">
       <c r="A249" s="5" t="s">
@@ -13568,12 +13595,12 @@
       </c>
     </row>
     <row r="254" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A254" s="17" t="s">
+      <c r="A254" s="20" t="s">
         <v>1160</v>
       </c>
-      <c r="B254" s="17"/>
-      <c r="C254" s="17"/>
-      <c r="D254" s="17"/>
+      <c r="B254" s="20"/>
+      <c r="C254" s="20"/>
+      <c r="D254" s="20"/>
     </row>
     <row r="255" spans="1:5">
       <c r="A255" s="5" t="s">
@@ -13618,12 +13645,12 @@
       </c>
     </row>
     <row r="259" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A259" s="17" t="s">
+      <c r="A259" s="20" t="s">
         <v>1166</v>
       </c>
-      <c r="B259" s="17"/>
-      <c r="C259" s="17"/>
-      <c r="D259" s="17"/>
+      <c r="B259" s="20"/>
+      <c r="C259" s="20"/>
+      <c r="D259" s="20"/>
     </row>
     <row r="260" spans="1:4" ht="26.4">
       <c r="A260" s="5" t="s">
@@ -13654,12 +13681,12 @@
       </c>
     </row>
     <row r="263" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A263" s="17" t="s">
+      <c r="A263" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B263" s="17"/>
-      <c r="C263" s="17"/>
-      <c r="D263" s="17"/>
+      <c r="B263" s="20"/>
+      <c r="C263" s="20"/>
+      <c r="D263" s="20"/>
     </row>
     <row r="264" spans="1:4" ht="55.2">
       <c r="A264" s="5" t="s">
@@ -13718,12 +13745,12 @@
       </c>
     </row>
     <row r="269" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A269" s="17" t="s">
+      <c r="A269" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B269" s="17"/>
-      <c r="C269" s="17"/>
-      <c r="D269" s="17"/>
+      <c r="B269" s="20"/>
+      <c r="C269" s="20"/>
+      <c r="D269" s="20"/>
     </row>
     <row r="270" spans="1:4">
       <c r="A270" s="5" t="s">
@@ -13782,23 +13809,23 @@
       </c>
     </row>
     <row r="276" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A276" s="27" t="s">
+      <c r="A276" s="29" t="s">
         <v>1185</v>
       </c>
-      <c r="B276" s="27"/>
-      <c r="C276" s="27"/>
-      <c r="D276" s="27"/>
+      <c r="B276" s="29"/>
+      <c r="C276" s="29"/>
+      <c r="D276" s="29"/>
       <c r="E276" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="277" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A277" s="17" t="s">
+      <c r="A277" s="20" t="s">
         <v>1186</v>
       </c>
-      <c r="B277" s="17"/>
-      <c r="C277" s="17"/>
-      <c r="D277" s="17"/>
+      <c r="B277" s="20"/>
+      <c r="C277" s="20"/>
+      <c r="D277" s="20"/>
     </row>
     <row r="278" spans="1:5" ht="41.4">
       <c r="A278" s="5" t="s">
@@ -13871,12 +13898,12 @@
       </c>
     </row>
     <row r="284" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A284" s="17" t="s">
+      <c r="A284" s="20" t="s">
         <v>1196</v>
       </c>
-      <c r="B284" s="17"/>
-      <c r="C284" s="17"/>
-      <c r="D284" s="17"/>
+      <c r="B284" s="20"/>
+      <c r="C284" s="20"/>
+      <c r="D284" s="20"/>
     </row>
     <row r="285" spans="1:5">
       <c r="A285" s="5" t="s">
@@ -14005,12 +14032,12 @@
       </c>
     </row>
     <row r="295" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A295" s="17" t="s">
+      <c r="A295" s="20" t="s">
         <v>1214</v>
       </c>
-      <c r="B295" s="17"/>
-      <c r="C295" s="17"/>
-      <c r="D295" s="17"/>
+      <c r="B295" s="20"/>
+      <c r="C295" s="20"/>
+      <c r="D295" s="20"/>
     </row>
     <row r="296" spans="1:4">
       <c r="A296" s="5" t="s">
@@ -14055,12 +14082,12 @@
       </c>
     </row>
     <row r="300" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A300" s="17" t="s">
+      <c r="A300" s="20" t="s">
         <v>1221</v>
       </c>
-      <c r="B300" s="17"/>
-      <c r="C300" s="17"/>
-      <c r="D300" s="17"/>
+      <c r="B300" s="20"/>
+      <c r="C300" s="20"/>
+      <c r="D300" s="20"/>
     </row>
     <row r="301" spans="1:4" ht="39.6">
       <c r="A301" s="5" t="s">
@@ -14119,12 +14146,12 @@
       </c>
     </row>
     <row r="306" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A306" s="17" t="s">
+      <c r="A306" s="20" t="s">
         <v>1229</v>
       </c>
-      <c r="B306" s="17"/>
-      <c r="C306" s="17"/>
-      <c r="D306" s="17"/>
+      <c r="B306" s="20"/>
+      <c r="C306" s="20"/>
+      <c r="D306" s="20"/>
     </row>
     <row r="307" spans="1:4">
       <c r="A307" s="5" t="s">
@@ -14267,12 +14294,12 @@
       </c>
     </row>
     <row r="318" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A318" s="17" t="s">
+      <c r="A318" s="20" t="s">
         <v>1248</v>
       </c>
-      <c r="B318" s="17"/>
-      <c r="C318" s="17"/>
-      <c r="D318" s="17"/>
+      <c r="B318" s="20"/>
+      <c r="C318" s="20"/>
+      <c r="D318" s="20"/>
     </row>
     <row r="319" spans="1:4" ht="27.6">
       <c r="A319" s="5" t="s">
@@ -14317,12 +14344,12 @@
       </c>
     </row>
     <row r="323" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A323" s="17" t="s">
+      <c r="A323" s="20" t="s">
         <v>862</v>
       </c>
-      <c r="B323" s="17"/>
-      <c r="C323" s="17"/>
-      <c r="D323" s="17"/>
+      <c r="B323" s="20"/>
+      <c r="C323" s="20"/>
+      <c r="D323" s="20"/>
     </row>
     <row r="324" spans="1:4">
       <c r="A324" s="5" t="s">
@@ -14367,12 +14394,12 @@
       </c>
     </row>
     <row r="328" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A328" s="17" t="s">
+      <c r="A328" s="20" t="s">
         <v>855</v>
       </c>
-      <c r="B328" s="17"/>
-      <c r="C328" s="17"/>
-      <c r="D328" s="17"/>
+      <c r="B328" s="20"/>
+      <c r="C328" s="20"/>
+      <c r="D328" s="20"/>
     </row>
     <row r="329" spans="1:4" ht="96.6">
       <c r="A329" s="5" t="s">
@@ -14446,6 +14473,61 @@
     </row>
   </sheetData>
   <mergeCells count="63">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A100:D100"/>
+    <mergeCell ref="A105:D105"/>
+    <mergeCell ref="A113:D113"/>
+    <mergeCell ref="A114:D114"/>
+    <mergeCell ref="A120:D120"/>
+    <mergeCell ref="A128:D128"/>
+    <mergeCell ref="A132:D132"/>
+    <mergeCell ref="A139:D139"/>
+    <mergeCell ref="A143:D143"/>
+    <mergeCell ref="A148:D148"/>
+    <mergeCell ref="A153:D153"/>
+    <mergeCell ref="A154:D154"/>
+    <mergeCell ref="A160:D160"/>
+    <mergeCell ref="A166:D166"/>
+    <mergeCell ref="A171:D171"/>
+    <mergeCell ref="A175:D175"/>
+    <mergeCell ref="A178:D178"/>
+    <mergeCell ref="A184:D184"/>
+    <mergeCell ref="A189:D189"/>
+    <mergeCell ref="A195:D195"/>
+    <mergeCell ref="A202:D202"/>
+    <mergeCell ref="A211:D211"/>
+    <mergeCell ref="A212:D212"/>
+    <mergeCell ref="A219:D219"/>
+    <mergeCell ref="A223:D223"/>
+    <mergeCell ref="A227:D227"/>
+    <mergeCell ref="A232:D232"/>
+    <mergeCell ref="A238:D238"/>
+    <mergeCell ref="A244:D244"/>
+    <mergeCell ref="A245:D245"/>
+    <mergeCell ref="A248:D248"/>
+    <mergeCell ref="A254:D254"/>
+    <mergeCell ref="A259:D259"/>
+    <mergeCell ref="A263:D263"/>
+    <mergeCell ref="A269:D269"/>
+    <mergeCell ref="A276:D276"/>
     <mergeCell ref="A318:D318"/>
     <mergeCell ref="A323:D323"/>
     <mergeCell ref="A328:D328"/>
@@ -14454,61 +14536,6 @@
     <mergeCell ref="A295:D295"/>
     <mergeCell ref="A300:D300"/>
     <mergeCell ref="A306:D306"/>
-    <mergeCell ref="A254:D254"/>
-    <mergeCell ref="A259:D259"/>
-    <mergeCell ref="A263:D263"/>
-    <mergeCell ref="A269:D269"/>
-    <mergeCell ref="A276:D276"/>
-    <mergeCell ref="A232:D232"/>
-    <mergeCell ref="A238:D238"/>
-    <mergeCell ref="A244:D244"/>
-    <mergeCell ref="A245:D245"/>
-    <mergeCell ref="A248:D248"/>
-    <mergeCell ref="A211:D211"/>
-    <mergeCell ref="A212:D212"/>
-    <mergeCell ref="A219:D219"/>
-    <mergeCell ref="A223:D223"/>
-    <mergeCell ref="A227:D227"/>
-    <mergeCell ref="A178:D178"/>
-    <mergeCell ref="A184:D184"/>
-    <mergeCell ref="A189:D189"/>
-    <mergeCell ref="A195:D195"/>
-    <mergeCell ref="A202:D202"/>
-    <mergeCell ref="A154:D154"/>
-    <mergeCell ref="A160:D160"/>
-    <mergeCell ref="A166:D166"/>
-    <mergeCell ref="A171:D171"/>
-    <mergeCell ref="A175:D175"/>
-    <mergeCell ref="A132:D132"/>
-    <mergeCell ref="A139:D139"/>
-    <mergeCell ref="A143:D143"/>
-    <mergeCell ref="A148:D148"/>
-    <mergeCell ref="A153:D153"/>
-    <mergeCell ref="A105:D105"/>
-    <mergeCell ref="A113:D113"/>
-    <mergeCell ref="A114:D114"/>
-    <mergeCell ref="A120:D120"/>
-    <mergeCell ref="A128:D128"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A83:D83"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="A100:D100"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -14528,101 +14555,101 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:5" ht="18">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="31" t="s">
         <v>1278</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="33" t="s">
         <v>1279</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="14" t="s">
         <v>1280</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="14" t="s">
         <v>1281</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="14" t="s">
         <v>655</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="14" t="s">
         <v>497</v>
       </c>
-      <c r="E5" s="31" t="s">
+      <c r="E5" s="14" t="s">
         <v>1282</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="43.2">
-      <c r="A6" s="32">
+    <row r="6" spans="1:5">
+      <c r="A6" s="15">
         <v>1</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="15" t="s">
         <v>1272</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-    </row>
-    <row r="7" spans="1:5" ht="100.8">
-      <c r="A7" s="32">
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+    </row>
+    <row r="7" spans="1:5" ht="28.8">
+      <c r="A7" s="15">
         <v>2</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="16" t="s">
         <v>1283</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="15" t="s">
         <v>1284</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="16" t="s">
         <v>1285</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="16" t="s">
         <v>1286</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="72">
-      <c r="A8" s="32">
+    <row r="8" spans="1:5" ht="28.8">
+      <c r="A8" s="15">
         <v>3</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="16" t="s">
         <v>1287</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="15" t="s">
         <v>1284</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="16" t="s">
         <v>1288</v>
       </c>
-      <c r="E8" s="33" t="s">
+      <c r="E8" s="16" t="s">
         <v>1289</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="33" t="s">
         <v>1290</v>
       </c>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="14" t="s">
         <v>1280</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="14" t="s">
         <v>1291</v>
       </c>
       <c r="C11" s="34" t="s">
@@ -14631,11 +14658,11 @@
       <c r="D11" s="35"/>
       <c r="E11" s="36"/>
     </row>
-    <row r="12" spans="1:5" ht="43.2">
-      <c r="A12" s="32">
+    <row r="12" spans="1:5">
+      <c r="A12" s="15">
         <v>1</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="16" t="s">
         <v>1292</v>
       </c>
       <c r="C12" s="37" t="s">
@@ -14645,8 +14672,8 @@
       <c r="E12" s="38"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="32"/>
-      <c r="B13" s="33"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="37" t="s">
         <v>1294</v>
       </c>
@@ -14665,12 +14692,199 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="C13:E13"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AFF2AF-D4BC-4BC0-A7E1-D98D2CA71943}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="6.88671875" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="90.88671875" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="21">
+      <c r="A1" s="39" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+    </row>
+    <row r="3" spans="1:4" ht="15.6">
+      <c r="A3" s="29" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+    </row>
+    <row r="5" spans="1:4" ht="138">
+      <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>831</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>832</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="82.8">
+      <c r="A6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>833</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>834</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="110.4">
+      <c r="A7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>835</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>836</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="165.6">
+      <c r="A8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>837</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>838</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="20" t="s">
+        <v>839</v>
+      </c>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" spans="1:4" ht="124.2">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>840</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>841</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="409.2">
+      <c r="A12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>842</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>843</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="151.80000000000001">
+      <c r="A13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>844</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>845</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="82.8">
+      <c r="A14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>846</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>847</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="220.8">
+      <c r="A15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>848</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="20" t="s">
+        <v>850</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
working onnbfc dashboard(aquire) part this part is divided into 5 steps verification ,offer,winner,agreement and e-nach, submit
</commit_message>
<xml_diff>
--- a/Itarang_Work_Report_3_Months_2026-05-25.xlsx
+++ b/Itarang_Work_Report_3_Months_2026-05-25.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55859C38-C20D-44B0-B831-FE0972B1A015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9F45A69-CBC6-4082-BE27-818841D98660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2628" uniqueCount="1301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2639" uniqueCount="1339">
   <si>
     <t>iTarang — 3-Month Work Report</t>
   </si>
@@ -3918,20 +3918,134 @@
     <t>Testing pending</t>
   </si>
   <si>
-    <t>5.  NBFC Addendum (V1 +V2)</t>
-  </si>
-  <si>
     <t>LIST OF CHANGES</t>
   </si>
   <si>
     <t>ZOHO Integration</t>
+  </si>
+  <si>
+    <t>pending</t>
+  </si>
+  <si>
+    <t>Daily task</t>
+  </si>
+  <si>
+    <t>1)</t>
+  </si>
+  <si>
+    <t>BRD POINTS</t>
+  </si>
+  <si>
+    <t>Lead capture (Step 1)</t>
+  </si>
+  <si>
+    <t>Two new fields: resident status (Owned/Rented) and existing insurance status (Health / Life, Yes/No).</t>
+  </si>
+  <si>
+    <t>Step 2 KYC</t>
+  </si>
+  <si>
+    <t>Structurally unchanged except consent-form content.</t>
+  </si>
+  <si>
+    <t>Admin KYC / BRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">consent some points are added </t>
+  </si>
+  <si>
+    <t>NBFC routing</t>
+  </si>
+  <si>
+    <t>Competitive. Customer picks up to 2 NBFCs; customer picks the winner.</t>
+  </si>
+  <si>
+    <t>loan product update</t>
+  </si>
+  <si>
+    <t xml:space="preserve">loan product and nbfc should be attach through the location(state,city) </t>
+  </si>
+  <si>
+    <t>Credit Bureau — Equifax</t>
+  </si>
+  <si>
+    <t>in kyc flow ,step 2 (customer kyc)</t>
+  </si>
+  <si>
+    <t>Product Selection — Section G (Financing Options)</t>
+  </si>
+  <si>
+    <t>1)Battery and charger photo uploads added to Sections B and C (serial close-up + unit photo).</t>
+  </si>
+  <si>
+    <t>2)removed admin side - "loan rejection","product rejection" removed this entitys</t>
+  </si>
+  <si>
+    <t>3) submit flow now changes - the lead flows into cometitive NBFC routing, not to an admin panel</t>
+  </si>
+  <si>
+    <t>5.  NBFC Addendum</t>
+  </si>
+  <si>
+    <t>Field investigation</t>
+  </si>
+  <si>
+    <t>video kyc</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>compleyted</t>
+  </si>
+  <si>
+    <t>Enach</t>
+  </si>
+  <si>
+    <t>Working</t>
+  </si>
+  <si>
+    <t>working</t>
+  </si>
+  <si>
+    <t>Acquire navbar</t>
+  </si>
+  <si>
+    <t>1) Aquire,monitor, recover sections added</t>
+  </si>
+  <si>
+    <t>Aquire - showing the BRE - and nbfc scheme (hold dealer details, status, info)</t>
+  </si>
+  <si>
+    <t>Todays Work</t>
+  </si>
+  <si>
+    <t>Call sumrit and ask to enable active vkyc</t>
+  </si>
+  <si>
+    <t>agreement initate button fixing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">production should be working </t>
+  </si>
+  <si>
+    <t>Remaining part of nbfc flow connect to kartik sir and move further with plan</t>
+  </si>
+  <si>
+    <t>enach flow</t>
+  </si>
+  <si>
+    <t>we have 2 option for video kyc 1)itarang vkyc,2)own work on own vkyc part</t>
+  </si>
+  <si>
+    <t>column connection of implemented part</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4008,8 +4122,34 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4086,8 +4226,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -4143,11 +4289,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBFC9D4"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBFC9D4"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBFC9D4"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFBFC9D4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4189,6 +4350,24 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -4197,9 +4376,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -4225,12 +4401,13 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4241,13 +4418,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4590,7 +4761,7 @@
   <sheetPr>
     <tabColor rgb="FF0F172A"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -4600,36 +4771,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
     </row>
     <row r="7" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
     </row>
     <row r="8" spans="1:5" ht="22.05" customHeight="1">
       <c r="A8" s="1" t="s">
@@ -4721,70 +4892,81 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
+        <v>1299</v>
+      </c>
+      <c r="E13" t="s">
         <v>1300</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A15" s="20" t="s">
+    <row r="14" spans="1:5">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="19.95" customHeight="1">
+      <c r="A22" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-    </row>
-    <row r="16" spans="1:5" ht="27.6">
-      <c r="A16" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+    </row>
+    <row r="23" spans="1:4" ht="27.6">
+      <c r="A23" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="27.6">
-      <c r="A17" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="7" t="s">
+      <c r="D23" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="27.6">
+      <c r="A24" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="27.6">
-      <c r="A18" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="7" t="s">
+      <c r="D24" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="27.6">
+      <c r="A25" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="D25" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D26" s="8" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4794,7 +4976,7 @@
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A22:D22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B8" location="#'Dealer Onboarding'!A1" tooltip="Open Dealer Onboarding tab" display="Dealer Onboarding" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -4823,34 +5005,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
@@ -4965,12 +5147,12 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
@@ -4987,23 +5169,23 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
       <c r="E18" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="5" t="s">
@@ -5076,12 +5258,12 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
     </row>
     <row r="27" spans="1:5" ht="27.6">
       <c r="A27" s="5" t="s">
@@ -5112,23 +5294,23 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
       <c r="E31" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A32" s="20" t="s">
+      <c r="A32" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
     </row>
     <row r="33" spans="1:4" ht="27.6">
       <c r="A33" s="5" t="s">
@@ -5187,12 +5369,12 @@
       </c>
     </row>
     <row r="38" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="24"/>
+      <c r="D38" s="24"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5" t="s">
@@ -5223,12 +5405,12 @@
       </c>
     </row>
     <row r="42" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A42" s="20" t="s">
+      <c r="A42" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="5" t="s">
@@ -5273,12 +5455,12 @@
       </c>
     </row>
     <row r="47" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A47" s="20" t="s">
+      <c r="A47" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="5" t="s">
@@ -5323,23 +5505,23 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A53" s="21" t="s">
+      <c r="A53" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="B53" s="21"/>
-      <c r="C53" s="21"/>
-      <c r="D53" s="21"/>
+      <c r="B53" s="28"/>
+      <c r="C53" s="28"/>
+      <c r="D53" s="28"/>
       <c r="E53" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A54" s="20" t="s">
+      <c r="A54" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="24"/>
+      <c r="D54" s="24"/>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
@@ -5370,12 +5552,12 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A58" s="20" t="s">
+      <c r="A58" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="B58" s="20"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
+      <c r="B58" s="24"/>
+      <c r="C58" s="24"/>
+      <c r="D58" s="24"/>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="5" t="s">
@@ -5434,23 +5616,23 @@
       </c>
     </row>
     <row r="65" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A65" s="21" t="s">
+      <c r="A65" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="B65" s="21"/>
-      <c r="C65" s="21"/>
-      <c r="D65" s="21"/>
+      <c r="B65" s="28"/>
+      <c r="C65" s="28"/>
+      <c r="D65" s="28"/>
       <c r="E65" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A66" s="20" t="s">
+      <c r="A66" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
+      <c r="B66" s="24"/>
+      <c r="C66" s="24"/>
+      <c r="D66" s="24"/>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="5" t="s">
@@ -5481,12 +5663,12 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A70" s="20" t="s">
+      <c r="A70" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="B70" s="20"/>
-      <c r="C70" s="20"/>
-      <c r="D70" s="20"/>
+      <c r="B70" s="24"/>
+      <c r="C70" s="24"/>
+      <c r="D70" s="24"/>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="5" t="s">
@@ -5531,12 +5713,12 @@
       </c>
     </row>
     <row r="75" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A75" s="20" t="s">
+      <c r="A75" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="B75" s="20"/>
-      <c r="C75" s="20"/>
-      <c r="D75" s="20"/>
+      <c r="B75" s="24"/>
+      <c r="C75" s="24"/>
+      <c r="D75" s="24"/>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" s="5" t="s">
@@ -5553,12 +5735,12 @@
       </c>
     </row>
     <row r="78" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A78" s="20" t="s">
+      <c r="A78" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="B78" s="20"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="24"/>
+      <c r="D78" s="24"/>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="5" t="s">
@@ -5589,12 +5771,12 @@
       </c>
     </row>
     <row r="82" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A82" s="20" t="s">
+      <c r="A82" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="B82" s="20"/>
-      <c r="C82" s="20"/>
-      <c r="D82" s="20"/>
+      <c r="B82" s="24"/>
+      <c r="C82" s="24"/>
+      <c r="D82" s="24"/>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="5" t="s">
@@ -5639,12 +5821,12 @@
       </c>
     </row>
     <row r="87" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A87" s="20" t="s">
+      <c r="A87" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="B87" s="20"/>
-      <c r="C87" s="20"/>
-      <c r="D87" s="20"/>
+      <c r="B87" s="24"/>
+      <c r="C87" s="24"/>
+      <c r="D87" s="24"/>
     </row>
     <row r="88" spans="1:5">
       <c r="A88" s="5" t="s">
@@ -5661,23 +5843,23 @@
       </c>
     </row>
     <row r="91" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A91" s="21" t="s">
+      <c r="A91" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="B91" s="21"/>
-      <c r="C91" s="21"/>
-      <c r="D91" s="21"/>
+      <c r="B91" s="28"/>
+      <c r="C91" s="28"/>
+      <c r="D91" s="28"/>
       <c r="E91" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A92" s="20" t="s">
+      <c r="A92" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="B92" s="20"/>
-      <c r="C92" s="20"/>
-      <c r="D92" s="20"/>
+      <c r="B92" s="24"/>
+      <c r="C92" s="24"/>
+      <c r="D92" s="24"/>
     </row>
     <row r="93" spans="1:5">
       <c r="A93" s="5" t="s">
@@ -5834,12 +6016,12 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A105" s="20" t="s">
+      <c r="A105" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B105" s="20"/>
-      <c r="C105" s="20"/>
-      <c r="D105" s="20"/>
+      <c r="B105" s="24"/>
+      <c r="C105" s="24"/>
+      <c r="D105" s="24"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="5" t="s">
@@ -5884,12 +6066,12 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A110" s="20" t="s">
+      <c r="A110" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="B110" s="20"/>
-      <c r="C110" s="20"/>
-      <c r="D110" s="20"/>
+      <c r="B110" s="24"/>
+      <c r="C110" s="24"/>
+      <c r="D110" s="24"/>
     </row>
     <row r="111" spans="1:4" ht="27.6">
       <c r="A111" s="5" t="s">
@@ -6010,34 +6192,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="31" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
       <c r="E4" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6057,12 +6239,12 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="24" t="s">
         <v>192</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
       <c r="E7" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6110,12 +6292,12 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="24" t="s">
         <v>199</v>
       </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
       <c r="E12" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6149,23 +6331,23 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="30" t="s">
         <v>204</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
       <c r="E17" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="24" t="s">
         <v>205</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
       <c r="E18" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6241,12 +6423,12 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
       <c r="E25" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6364,12 +6546,12 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A35" s="20" t="s">
+      <c r="A35" s="24" t="s">
         <v>233</v>
       </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
       <c r="E35" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6459,12 +6641,12 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A43" s="20" t="s">
+      <c r="A43" s="24" t="s">
         <v>246</v>
       </c>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
       <c r="E43" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6596,12 +6778,12 @@
       </c>
     </row>
     <row r="54" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A54" s="20" t="s">
+      <c r="A54" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="24"/>
+      <c r="D54" s="24"/>
       <c r="E54" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6649,12 +6831,12 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A59" s="20" t="s">
+      <c r="A59" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="B59" s="20"/>
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
+      <c r="B59" s="24"/>
+      <c r="C59" s="24"/>
+      <c r="D59" s="24"/>
       <c r="E59" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6800,12 +6982,12 @@
       </c>
     </row>
     <row r="71" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A71" s="20" t="s">
+      <c r="A71" s="24" t="s">
         <v>293</v>
       </c>
-      <c r="B71" s="20"/>
-      <c r="C71" s="20"/>
-      <c r="D71" s="20"/>
+      <c r="B71" s="24"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="24"/>
       <c r="E71" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6951,12 +7133,12 @@
       </c>
     </row>
     <row r="83" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A83" s="20" t="s">
+      <c r="A83" s="24" t="s">
         <v>314</v>
       </c>
-      <c r="B83" s="20"/>
-      <c r="C83" s="20"/>
-      <c r="D83" s="20"/>
+      <c r="B83" s="24"/>
+      <c r="C83" s="24"/>
+      <c r="D83" s="24"/>
       <c r="E83" s="10" t="s">
         <v>1272</v>
       </c>
@@ -6976,12 +7158,12 @@
       </c>
     </row>
     <row r="86" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A86" s="20" t="s">
+      <c r="A86" s="24" t="s">
         <v>317</v>
       </c>
-      <c r="B86" s="20"/>
-      <c r="C86" s="20"/>
-      <c r="D86" s="20"/>
+      <c r="B86" s="24"/>
+      <c r="C86" s="24"/>
+      <c r="D86" s="24"/>
       <c r="E86" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7071,12 +7253,12 @@
       </c>
     </row>
     <row r="94" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A94" s="20" t="s">
+      <c r="A94" s="24" t="s">
         <v>331</v>
       </c>
-      <c r="B94" s="20"/>
-      <c r="C94" s="20"/>
-      <c r="D94" s="20"/>
+      <c r="B94" s="24"/>
+      <c r="C94" s="24"/>
+      <c r="D94" s="24"/>
       <c r="E94" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7152,12 +7334,12 @@
       </c>
     </row>
     <row r="101" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A101" s="20" t="s">
+      <c r="A101" s="24" t="s">
         <v>342</v>
       </c>
-      <c r="B101" s="20"/>
-      <c r="C101" s="20"/>
-      <c r="D101" s="20"/>
+      <c r="B101" s="24"/>
+      <c r="C101" s="24"/>
+      <c r="D101" s="24"/>
       <c r="E101" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7275,12 +7457,12 @@
       </c>
     </row>
     <row r="111" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A111" s="20" t="s">
+      <c r="A111" s="24" t="s">
         <v>361</v>
       </c>
-      <c r="B111" s="20"/>
-      <c r="C111" s="20"/>
-      <c r="D111" s="20"/>
+      <c r="B111" s="24"/>
+      <c r="C111" s="24"/>
+      <c r="D111" s="24"/>
       <c r="E111" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7496,23 +7678,23 @@
       </c>
     </row>
     <row r="129" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A129" s="23" t="s">
+      <c r="A129" s="30" t="s">
         <v>392</v>
       </c>
-      <c r="B129" s="23"/>
-      <c r="C129" s="23"/>
-      <c r="D129" s="23"/>
+      <c r="B129" s="30"/>
+      <c r="C129" s="30"/>
+      <c r="D129" s="30"/>
       <c r="E129" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="130" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A130" s="20" t="s">
+      <c r="A130" s="24" t="s">
         <v>393</v>
       </c>
-      <c r="B130" s="20"/>
-      <c r="C130" s="20"/>
-      <c r="D130" s="20"/>
+      <c r="B130" s="24"/>
+      <c r="C130" s="24"/>
+      <c r="D130" s="24"/>
     </row>
     <row r="131" spans="1:5" ht="27.6">
       <c r="A131" s="5" t="s">
@@ -7837,12 +8019,12 @@
       </c>
     </row>
     <row r="155" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A155" s="20" t="s">
+      <c r="A155" s="24" t="s">
         <v>440</v>
       </c>
-      <c r="B155" s="20"/>
-      <c r="C155" s="20"/>
-      <c r="D155" s="20"/>
+      <c r="B155" s="24"/>
+      <c r="C155" s="24"/>
+      <c r="D155" s="24"/>
       <c r="E155" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7918,12 +8100,12 @@
       </c>
     </row>
     <row r="162" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A162" s="20" t="s">
+      <c r="A162" s="24" t="s">
         <v>451</v>
       </c>
-      <c r="B162" s="20"/>
-      <c r="C162" s="20"/>
-      <c r="D162" s="20"/>
+      <c r="B162" s="24"/>
+      <c r="C162" s="24"/>
+      <c r="D162" s="24"/>
       <c r="E162" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7957,12 +8139,12 @@
       </c>
     </row>
     <row r="166" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A166" s="20" t="s">
+      <c r="A166" s="24" t="s">
         <v>456</v>
       </c>
-      <c r="B166" s="20"/>
-      <c r="C166" s="20"/>
-      <c r="D166" s="20"/>
+      <c r="B166" s="24"/>
+      <c r="C166" s="24"/>
+      <c r="D166" s="24"/>
       <c r="E166" s="10" t="s">
         <v>1272</v>
       </c>
@@ -7996,12 +8178,12 @@
       </c>
     </row>
     <row r="170" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A170" s="20" t="s">
+      <c r="A170" s="24" t="s">
         <v>459</v>
       </c>
-      <c r="B170" s="20"/>
-      <c r="C170" s="20"/>
-      <c r="D170" s="20"/>
+      <c r="B170" s="24"/>
+      <c r="C170" s="24"/>
+      <c r="D170" s="24"/>
       <c r="E170" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8035,12 +8217,12 @@
       </c>
     </row>
     <row r="174" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A174" s="20" t="s">
+      <c r="A174" s="24" t="s">
         <v>462</v>
       </c>
-      <c r="B174" s="20"/>
-      <c r="C174" s="20"/>
-      <c r="D174" s="20"/>
+      <c r="B174" s="24"/>
+      <c r="C174" s="24"/>
+      <c r="D174" s="24"/>
       <c r="E174" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8116,12 +8298,12 @@
       </c>
     </row>
     <row r="181" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A181" s="20" t="s">
+      <c r="A181" s="24" t="s">
         <v>473</v>
       </c>
-      <c r="B181" s="20"/>
-      <c r="C181" s="20"/>
-      <c r="D181" s="20"/>
+      <c r="B181" s="24"/>
+      <c r="C181" s="24"/>
+      <c r="D181" s="24"/>
       <c r="E181" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8183,12 +8365,12 @@
       </c>
     </row>
     <row r="187" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A187" s="20" t="s">
+      <c r="A187" s="24" t="s">
         <v>482</v>
       </c>
-      <c r="B187" s="20"/>
-      <c r="C187" s="20"/>
-      <c r="D187" s="20"/>
+      <c r="B187" s="24"/>
+      <c r="C187" s="24"/>
+      <c r="D187" s="24"/>
       <c r="E187" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8264,12 +8446,12 @@
       </c>
     </row>
     <row r="194" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A194" s="20" t="s">
+      <c r="A194" s="24" t="s">
         <v>492</v>
       </c>
-      <c r="B194" s="20"/>
-      <c r="C194" s="20"/>
-      <c r="D194" s="20"/>
+      <c r="B194" s="24"/>
+      <c r="C194" s="24"/>
+      <c r="D194" s="24"/>
       <c r="E194" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8423,34 +8605,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="33" t="s">
         <v>506</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="32" t="s">
         <v>507</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="24" t="s">
         <v>508</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:5" ht="27.6">
       <c r="A5" s="5" t="s">
@@ -8523,12 +8705,12 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="24" t="s">
         <v>519</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
       <c r="E11" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8604,12 +8786,12 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="24" t="s">
         <v>528</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
       <c r="E18" s="10" t="s">
         <v>1272</v>
       </c>
@@ -8923,12 +9105,12 @@
       </c>
     </row>
     <row r="42" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A42" s="20" t="s">
+      <c r="A42" s="24" t="s">
         <v>573</v>
       </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
       <c r="E42" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9060,12 +9242,12 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A53" s="20" t="s">
+      <c r="A53" s="24" t="s">
         <v>590</v>
       </c>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
+      <c r="B53" s="24"/>
+      <c r="C53" s="24"/>
+      <c r="D53" s="24"/>
       <c r="E53" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9225,12 +9407,12 @@
       </c>
     </row>
     <row r="66" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A66" s="20" t="s">
+      <c r="A66" s="24" t="s">
         <v>613</v>
       </c>
-      <c r="B66" s="20"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
+      <c r="B66" s="24"/>
+      <c r="C66" s="24"/>
+      <c r="D66" s="24"/>
       <c r="E66" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9306,12 +9488,12 @@
       </c>
     </row>
     <row r="73" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A73" s="20" t="s">
+      <c r="A73" s="24" t="s">
         <v>624</v>
       </c>
-      <c r="B73" s="20"/>
-      <c r="C73" s="20"/>
-      <c r="D73" s="20"/>
+      <c r="B73" s="24"/>
+      <c r="C73" s="24"/>
+      <c r="D73" s="24"/>
       <c r="E73" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9415,12 +9597,12 @@
       </c>
     </row>
     <row r="82" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A82" s="20" t="s">
+      <c r="A82" s="24" t="s">
         <v>639</v>
       </c>
-      <c r="B82" s="20"/>
-      <c r="C82" s="20"/>
-      <c r="D82" s="20"/>
+      <c r="B82" s="24"/>
+      <c r="C82" s="24"/>
+      <c r="D82" s="24"/>
       <c r="E82" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9524,12 +9706,12 @@
       </c>
     </row>
     <row r="91" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A91" s="20" t="s">
+      <c r="A91" s="24" t="s">
         <v>654</v>
       </c>
-      <c r="B91" s="20"/>
-      <c r="C91" s="20"/>
-      <c r="D91" s="20"/>
+      <c r="B91" s="24"/>
+      <c r="C91" s="24"/>
+      <c r="D91" s="24"/>
       <c r="E91" s="11" t="s">
         <v>1273</v>
       </c>
@@ -9604,7 +9786,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="66">
+    <row r="97" spans="1:5" ht="52.8">
       <c r="A97" s="5" t="s">
         <v>25</v>
       </c>
@@ -9759,12 +9941,12 @@
       </c>
     </row>
     <row r="109" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A109" s="20" t="s">
+      <c r="A109" s="24" t="s">
         <v>687</v>
       </c>
-      <c r="B109" s="20"/>
-      <c r="C109" s="20"/>
-      <c r="D109" s="20"/>
+      <c r="B109" s="24"/>
+      <c r="C109" s="24"/>
+      <c r="D109" s="24"/>
       <c r="E109" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9840,12 +10022,12 @@
       </c>
     </row>
     <row r="116" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A116" s="20" t="s">
+      <c r="A116" s="24" t="s">
         <v>696</v>
       </c>
-      <c r="B116" s="20"/>
-      <c r="C116" s="20"/>
-      <c r="D116" s="20"/>
+      <c r="B116" s="24"/>
+      <c r="C116" s="24"/>
+      <c r="D116" s="24"/>
       <c r="E116" s="10" t="s">
         <v>1272</v>
       </c>
@@ -9949,23 +10131,23 @@
       </c>
     </row>
     <row r="126" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A126" s="25" t="s">
+      <c r="A126" s="32" t="s">
         <v>708</v>
       </c>
-      <c r="B126" s="25"/>
-      <c r="C126" s="25"/>
-      <c r="D126" s="25"/>
+      <c r="B126" s="32"/>
+      <c r="C126" s="32"/>
+      <c r="D126" s="32"/>
       <c r="E126" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="128" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A128" s="20" t="s">
+      <c r="A128" s="24" t="s">
         <v>709</v>
       </c>
-      <c r="B128" s="20"/>
-      <c r="C128" s="20"/>
-      <c r="D128" s="20"/>
+      <c r="B128" s="24"/>
+      <c r="C128" s="24"/>
+      <c r="D128" s="24"/>
     </row>
     <row r="129" spans="1:4" ht="27.6">
       <c r="A129" s="5" t="s">
@@ -10035,34 +10217,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="35" t="s">
         <v>714</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="34" t="s">
         <v>715</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
       <c r="E3" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="24" t="s">
         <v>716</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
@@ -10135,12 +10317,12 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="24" t="s">
         <v>726</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
@@ -10171,12 +10353,12 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="24" t="s">
         <v>731</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="5" t="s">
@@ -10193,12 +10375,12 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="24" t="s">
         <v>734</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="5" t="s">
@@ -10257,12 +10439,12 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="24" t="s">
         <v>743</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="5" t="s">
@@ -10307,12 +10489,12 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="24" t="s">
         <v>749</v>
       </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5" t="s">
@@ -10357,23 +10539,23 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="34" t="s">
         <v>756</v>
       </c>
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
       <c r="E35" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A36" s="20" t="s">
+      <c r="A36" s="24" t="s">
         <v>757</v>
       </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="24"/>
+      <c r="D36" s="24"/>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="5" t="s">
@@ -10502,12 +10684,12 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A47" s="20" t="s">
+      <c r="A47" s="24" t="s">
         <v>768</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="5" t="s">
@@ -10552,23 +10734,23 @@
       </c>
     </row>
     <row r="53" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A53" s="27" t="s">
+      <c r="A53" s="34" t="s">
         <v>775</v>
       </c>
-      <c r="B53" s="27"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="27"/>
+      <c r="B53" s="34"/>
+      <c r="C53" s="34"/>
+      <c r="D53" s="34"/>
       <c r="E53" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A54" s="20" t="s">
+      <c r="A54" s="24" t="s">
         <v>776</v>
       </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="24"/>
+      <c r="D54" s="24"/>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="5" t="s">
@@ -10613,12 +10795,12 @@
       </c>
     </row>
     <row r="59" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A59" s="20" t="s">
+      <c r="A59" s="24" t="s">
         <v>783</v>
       </c>
-      <c r="B59" s="20"/>
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
+      <c r="B59" s="24"/>
+      <c r="C59" s="24"/>
+      <c r="D59" s="24"/>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="5" t="s">
@@ -10663,12 +10845,12 @@
       </c>
     </row>
     <row r="64" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A64" s="20" t="s">
+      <c r="A64" s="24" t="s">
         <v>788</v>
       </c>
-      <c r="B64" s="20"/>
-      <c r="C64" s="20"/>
-      <c r="D64" s="20"/>
+      <c r="B64" s="24"/>
+      <c r="C64" s="24"/>
+      <c r="D64" s="24"/>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="5" t="s">
@@ -10713,23 +10895,23 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A70" s="27" t="s">
+      <c r="A70" s="34" t="s">
         <v>794</v>
       </c>
-      <c r="B70" s="27"/>
-      <c r="C70" s="27"/>
-      <c r="D70" s="27"/>
+      <c r="B70" s="34"/>
+      <c r="C70" s="34"/>
+      <c r="D70" s="34"/>
       <c r="E70" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A71" s="20" t="s">
+      <c r="A71" s="24" t="s">
         <v>795</v>
       </c>
-      <c r="B71" s="20"/>
-      <c r="C71" s="20"/>
-      <c r="D71" s="20"/>
+      <c r="B71" s="24"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="24"/>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="5" t="s">
@@ -10802,12 +10984,12 @@
       </c>
     </row>
     <row r="78" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A78" s="20" t="s">
+      <c r="A78" s="24" t="s">
         <v>806</v>
       </c>
-      <c r="B78" s="20"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="24"/>
+      <c r="D78" s="24"/>
     </row>
     <row r="79" spans="1:5" ht="27.6">
       <c r="A79" s="5" t="s">
@@ -10824,12 +11006,12 @@
       </c>
     </row>
     <row r="81" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A81" s="20" t="s">
+      <c r="A81" s="24" t="s">
         <v>809</v>
       </c>
-      <c r="B81" s="20"/>
-      <c r="C81" s="20"/>
-      <c r="D81" s="20"/>
+      <c r="B81" s="24"/>
+      <c r="C81" s="24"/>
+      <c r="D81" s="24"/>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="5" t="s">
@@ -10874,23 +11056,23 @@
       </c>
     </row>
     <row r="87" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A87" s="27" t="s">
+      <c r="A87" s="34" t="s">
         <v>816</v>
       </c>
-      <c r="B87" s="27"/>
-      <c r="C87" s="27"/>
-      <c r="D87" s="27"/>
+      <c r="B87" s="34"/>
+      <c r="C87" s="34"/>
+      <c r="D87" s="34"/>
       <c r="E87" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A88" s="20" t="s">
+      <c r="A88" s="24" t="s">
         <v>817</v>
       </c>
-      <c r="B88" s="20"/>
-      <c r="C88" s="20"/>
-      <c r="D88" s="20"/>
+      <c r="B88" s="24"/>
+      <c r="C88" s="24"/>
+      <c r="D88" s="24"/>
     </row>
     <row r="89" spans="1:5">
       <c r="A89" s="5" t="s">
@@ -10935,12 +11117,12 @@
       </c>
     </row>
     <row r="93" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A93" s="20" t="s">
+      <c r="A93" s="24" t="s">
         <v>823</v>
       </c>
-      <c r="B93" s="20"/>
-      <c r="C93" s="20"/>
-      <c r="D93" s="20"/>
+      <c r="B93" s="24"/>
+      <c r="C93" s="24"/>
+      <c r="D93" s="24"/>
     </row>
     <row r="94" spans="1:5">
       <c r="A94" s="5" t="s">
@@ -11015,34 +11197,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>828</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
       <c r="E1" s="10" t="s">
         <v>1271</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="23" t="s">
         <v>829</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="24" t="s">
         <v>830</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
@@ -11101,12 +11283,12 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="24" t="s">
         <v>839</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
@@ -11179,12 +11361,12 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="24" t="s">
         <v>850</v>
       </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
     </row>
     <row r="18" spans="1:5" ht="39.6">
       <c r="A18" s="5" t="s">
@@ -11215,12 +11397,12 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
     </row>
     <row r="22" spans="1:5" ht="55.2">
       <c r="A22" s="5" t="s">
@@ -11251,12 +11433,12 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
     </row>
     <row r="26" spans="1:5" ht="27.6">
       <c r="A26" s="5" t="s">
@@ -11273,23 +11455,23 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="23" t="s">
         <v>865</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
       <c r="E29" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="24" t="s">
         <v>866</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="5" t="s">
@@ -11446,12 +11628,12 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A43" s="20" t="s">
+      <c r="A43" s="24" t="s">
         <v>888</v>
       </c>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
     </row>
     <row r="44" spans="1:4" ht="27.6">
       <c r="A44" s="5" t="s">
@@ -11524,12 +11706,12 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A50" s="20" t="s">
+      <c r="A50" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="24"/>
     </row>
     <row r="51" spans="1:5" ht="41.4">
       <c r="A51" s="5" t="s">
@@ -11574,12 +11756,12 @@
       </c>
     </row>
     <row r="55" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A55" s="20" t="s">
+      <c r="A55" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
+      <c r="B55" s="24"/>
+      <c r="C55" s="24"/>
+      <c r="D55" s="24"/>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="5" t="s">
@@ -11610,23 +11792,23 @@
       </c>
     </row>
     <row r="60" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A60" s="29" t="s">
+      <c r="A60" s="23" t="s">
         <v>909</v>
       </c>
-      <c r="B60" s="29"/>
-      <c r="C60" s="29"/>
-      <c r="D60" s="29"/>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
+      <c r="D60" s="23"/>
       <c r="E60" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A61" s="20" t="s">
+      <c r="A61" s="24" t="s">
         <v>910</v>
       </c>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
+      <c r="B61" s="24"/>
+      <c r="C61" s="24"/>
+      <c r="D61" s="24"/>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="5" t="s">
@@ -11685,12 +11867,12 @@
       </c>
     </row>
     <row r="67" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A67" s="20" t="s">
+      <c r="A67" s="24" t="s">
         <v>919</v>
       </c>
-      <c r="B67" s="20"/>
-      <c r="C67" s="20"/>
-      <c r="D67" s="20"/>
+      <c r="B67" s="24"/>
+      <c r="C67" s="24"/>
+      <c r="D67" s="24"/>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="5" t="s">
@@ -11763,12 +11945,12 @@
       </c>
     </row>
     <row r="74" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A74" s="20" t="s">
+      <c r="A74" s="24" t="s">
         <v>891</v>
       </c>
-      <c r="B74" s="20"/>
-      <c r="C74" s="20"/>
-      <c r="D74" s="20"/>
+      <c r="B74" s="24"/>
+      <c r="C74" s="24"/>
+      <c r="D74" s="24"/>
     </row>
     <row r="75" spans="1:4" ht="26.4">
       <c r="A75" s="5" t="s">
@@ -11869,12 +12051,12 @@
       </c>
     </row>
     <row r="83" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A83" s="20" t="s">
+      <c r="A83" s="24" t="s">
         <v>943</v>
       </c>
-      <c r="B83" s="20"/>
-      <c r="C83" s="20"/>
-      <c r="D83" s="20"/>
+      <c r="B83" s="24"/>
+      <c r="C83" s="24"/>
+      <c r="D83" s="24"/>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="5" t="s">
@@ -11961,12 +12143,12 @@
       </c>
     </row>
     <row r="91" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A91" s="20" t="s">
+      <c r="A91" s="24" t="s">
         <v>956</v>
       </c>
-      <c r="B91" s="20"/>
-      <c r="C91" s="20"/>
-      <c r="D91" s="20"/>
+      <c r="B91" s="24"/>
+      <c r="C91" s="24"/>
+      <c r="D91" s="24"/>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="5" t="s">
@@ -12025,12 +12207,12 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A97" s="20" t="s">
+      <c r="A97" s="24" t="s">
         <v>964</v>
       </c>
-      <c r="B97" s="20"/>
-      <c r="C97" s="20"/>
-      <c r="D97" s="20"/>
+      <c r="B97" s="24"/>
+      <c r="C97" s="24"/>
+      <c r="D97" s="24"/>
     </row>
     <row r="98" spans="1:4" ht="27.6">
       <c r="A98" s="5" t="s">
@@ -12047,12 +12229,12 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A100" s="20" t="s">
+      <c r="A100" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B100" s="20"/>
-      <c r="C100" s="20"/>
-      <c r="D100" s="20"/>
+      <c r="B100" s="24"/>
+      <c r="C100" s="24"/>
+      <c r="D100" s="24"/>
     </row>
     <row r="101" spans="1:4" ht="96.6">
       <c r="A101" s="5" t="s">
@@ -12097,12 +12279,12 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A105" s="20" t="s">
+      <c r="A105" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B105" s="20"/>
-      <c r="C105" s="20"/>
-      <c r="D105" s="20"/>
+      <c r="B105" s="24"/>
+      <c r="C105" s="24"/>
+      <c r="D105" s="24"/>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="5" t="s">
@@ -12175,23 +12357,23 @@
       </c>
     </row>
     <row r="113" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A113" s="29" t="s">
+      <c r="A113" s="23" t="s">
         <v>983</v>
       </c>
-      <c r="B113" s="29"/>
-      <c r="C113" s="29"/>
-      <c r="D113" s="29"/>
+      <c r="B113" s="23"/>
+      <c r="C113" s="23"/>
+      <c r="D113" s="23"/>
       <c r="E113" s="11" t="s">
         <v>1273</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A114" s="20" t="s">
+      <c r="A114" s="24" t="s">
         <v>984</v>
       </c>
-      <c r="B114" s="20"/>
-      <c r="C114" s="20"/>
-      <c r="D114" s="20"/>
+      <c r="B114" s="24"/>
+      <c r="C114" s="24"/>
+      <c r="D114" s="24"/>
     </row>
     <row r="115" spans="1:5">
       <c r="A115" s="5" t="s">
@@ -12250,12 +12432,12 @@
       </c>
     </row>
     <row r="120" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A120" s="20" t="s">
+      <c r="A120" s="24" t="s">
         <v>993</v>
       </c>
-      <c r="B120" s="20"/>
-      <c r="C120" s="20"/>
-      <c r="D120" s="20"/>
+      <c r="B120" s="24"/>
+      <c r="C120" s="24"/>
+      <c r="D120" s="24"/>
     </row>
     <row r="121" spans="1:5">
       <c r="A121" s="5" t="s">
@@ -12342,12 +12524,12 @@
       </c>
     </row>
     <row r="128" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A128" s="20" t="s">
+      <c r="A128" s="24" t="s">
         <v>1006</v>
       </c>
-      <c r="B128" s="20"/>
-      <c r="C128" s="20"/>
-      <c r="D128" s="20"/>
+      <c r="B128" s="24"/>
+      <c r="C128" s="24"/>
+      <c r="D128" s="24"/>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="5" t="s">
@@ -12378,12 +12560,12 @@
       </c>
     </row>
     <row r="132" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A132" s="20" t="s">
+      <c r="A132" s="24" t="s">
         <v>1011</v>
       </c>
-      <c r="B132" s="20"/>
-      <c r="C132" s="20"/>
-      <c r="D132" s="20"/>
+      <c r="B132" s="24"/>
+      <c r="C132" s="24"/>
+      <c r="D132" s="24"/>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="5" t="s">
@@ -12456,12 +12638,12 @@
       </c>
     </row>
     <row r="139" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A139" s="20" t="s">
+      <c r="A139" s="24" t="s">
         <v>1019</v>
       </c>
-      <c r="B139" s="20"/>
-      <c r="C139" s="20"/>
-      <c r="D139" s="20"/>
+      <c r="B139" s="24"/>
+      <c r="C139" s="24"/>
+      <c r="D139" s="24"/>
     </row>
     <row r="140" spans="1:4" ht="39.6">
       <c r="A140" s="5" t="s">
@@ -12492,12 +12674,12 @@
       </c>
     </row>
     <row r="143" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A143" s="20" t="s">
+      <c r="A143" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B143" s="20"/>
-      <c r="C143" s="20"/>
-      <c r="D143" s="20"/>
+      <c r="B143" s="24"/>
+      <c r="C143" s="24"/>
+      <c r="D143" s="24"/>
     </row>
     <row r="144" spans="1:4" ht="69">
       <c r="A144" s="5" t="s">
@@ -12542,12 +12724,12 @@
       </c>
     </row>
     <row r="148" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A148" s="20" t="s">
+      <c r="A148" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B148" s="20"/>
-      <c r="C148" s="20"/>
-      <c r="D148" s="20"/>
+      <c r="B148" s="24"/>
+      <c r="C148" s="24"/>
+      <c r="D148" s="24"/>
     </row>
     <row r="149" spans="1:5">
       <c r="A149" s="5" t="s">
@@ -12578,23 +12760,23 @@
       </c>
     </row>
     <row r="153" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A153" s="29" t="s">
+      <c r="A153" s="23" t="s">
         <v>1033</v>
       </c>
-      <c r="B153" s="29"/>
-      <c r="C153" s="29"/>
-      <c r="D153" s="29"/>
+      <c r="B153" s="23"/>
+      <c r="C153" s="23"/>
+      <c r="D153" s="23"/>
       <c r="E153" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="154" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A154" s="20" t="s">
+      <c r="A154" s="24" t="s">
         <v>1034</v>
       </c>
-      <c r="B154" s="20"/>
-      <c r="C154" s="20"/>
-      <c r="D154" s="20"/>
+      <c r="B154" s="24"/>
+      <c r="C154" s="24"/>
+      <c r="D154" s="24"/>
     </row>
     <row r="155" spans="1:5" ht="26.4">
       <c r="A155" s="5" t="s">
@@ -12653,12 +12835,12 @@
       </c>
     </row>
     <row r="160" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A160" s="20" t="s">
+      <c r="A160" s="24" t="s">
         <v>1043</v>
       </c>
-      <c r="B160" s="20"/>
-      <c r="C160" s="20"/>
-      <c r="D160" s="20"/>
+      <c r="B160" s="24"/>
+      <c r="C160" s="24"/>
+      <c r="D160" s="24"/>
     </row>
     <row r="161" spans="1:4" ht="27.6">
       <c r="A161" s="5" t="s">
@@ -12717,12 +12899,12 @@
       </c>
     </row>
     <row r="166" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A166" s="20" t="s">
+      <c r="A166" s="24" t="s">
         <v>1052</v>
       </c>
-      <c r="B166" s="20"/>
-      <c r="C166" s="20"/>
-      <c r="D166" s="20"/>
+      <c r="B166" s="24"/>
+      <c r="C166" s="24"/>
+      <c r="D166" s="24"/>
     </row>
     <row r="167" spans="1:4" ht="26.4">
       <c r="A167" s="5" t="s">
@@ -12767,12 +12949,12 @@
       </c>
     </row>
     <row r="171" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A171" s="20" t="s">
+      <c r="A171" s="24" t="s">
         <v>1058</v>
       </c>
-      <c r="B171" s="20"/>
-      <c r="C171" s="20"/>
-      <c r="D171" s="20"/>
+      <c r="B171" s="24"/>
+      <c r="C171" s="24"/>
+      <c r="D171" s="24"/>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="5" t="s">
@@ -12803,12 +12985,12 @@
       </c>
     </row>
     <row r="175" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A175" s="20" t="s">
+      <c r="A175" s="24" t="s">
         <v>1063</v>
       </c>
-      <c r="B175" s="20"/>
-      <c r="C175" s="20"/>
-      <c r="D175" s="20"/>
+      <c r="B175" s="24"/>
+      <c r="C175" s="24"/>
+      <c r="D175" s="24"/>
     </row>
     <row r="176" spans="1:4" ht="27.6">
       <c r="A176" s="5" t="s">
@@ -12825,12 +13007,12 @@
       </c>
     </row>
     <row r="178" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A178" s="20" t="s">
+      <c r="A178" s="24" t="s">
         <v>1066</v>
       </c>
-      <c r="B178" s="20"/>
-      <c r="C178" s="20"/>
-      <c r="D178" s="20"/>
+      <c r="B178" s="24"/>
+      <c r="C178" s="24"/>
+      <c r="D178" s="24"/>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" s="5" t="s">
@@ -12889,12 +13071,12 @@
       </c>
     </row>
     <row r="184" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A184" s="20" t="s">
+      <c r="A184" s="24" t="s">
         <v>1075</v>
       </c>
-      <c r="B184" s="20"/>
-      <c r="C184" s="20"/>
-      <c r="D184" s="20"/>
+      <c r="B184" s="24"/>
+      <c r="C184" s="24"/>
+      <c r="D184" s="24"/>
     </row>
     <row r="185" spans="1:4">
       <c r="A185" s="5" t="s">
@@ -12939,12 +13121,12 @@
       </c>
     </row>
     <row r="189" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A189" s="20" t="s">
+      <c r="A189" s="24" t="s">
         <v>1081</v>
       </c>
-      <c r="B189" s="20"/>
-      <c r="C189" s="20"/>
-      <c r="D189" s="20"/>
+      <c r="B189" s="24"/>
+      <c r="C189" s="24"/>
+      <c r="D189" s="24"/>
     </row>
     <row r="190" spans="1:4" ht="39.6">
       <c r="A190" s="5" t="s">
@@ -13003,12 +13185,12 @@
       </c>
     </row>
     <row r="195" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A195" s="20" t="s">
+      <c r="A195" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B195" s="20"/>
-      <c r="C195" s="20"/>
-      <c r="D195" s="20"/>
+      <c r="B195" s="24"/>
+      <c r="C195" s="24"/>
+      <c r="D195" s="24"/>
     </row>
     <row r="196" spans="1:4" ht="55.2">
       <c r="A196" s="5" t="s">
@@ -13081,12 +13263,12 @@
       </c>
     </row>
     <row r="202" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A202" s="20" t="s">
+      <c r="A202" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B202" s="20"/>
-      <c r="C202" s="20"/>
-      <c r="D202" s="20"/>
+      <c r="B202" s="24"/>
+      <c r="C202" s="24"/>
+      <c r="D202" s="24"/>
     </row>
     <row r="203" spans="1:4">
       <c r="A203" s="5" t="s">
@@ -13173,23 +13355,23 @@
       </c>
     </row>
     <row r="211" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A211" s="29" t="s">
+      <c r="A211" s="23" t="s">
         <v>1111</v>
       </c>
-      <c r="B211" s="29"/>
-      <c r="C211" s="29"/>
-      <c r="D211" s="29"/>
+      <c r="B211" s="23"/>
+      <c r="C211" s="23"/>
+      <c r="D211" s="23"/>
       <c r="E211" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="212" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A212" s="20" t="s">
+      <c r="A212" s="24" t="s">
         <v>1112</v>
       </c>
-      <c r="B212" s="20"/>
-      <c r="C212" s="20"/>
-      <c r="D212" s="20"/>
+      <c r="B212" s="24"/>
+      <c r="C212" s="24"/>
+      <c r="D212" s="24"/>
     </row>
     <row r="213" spans="1:5">
       <c r="A213" s="5" t="s">
@@ -13262,12 +13444,12 @@
       </c>
     </row>
     <row r="219" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A219" s="20" t="s">
+      <c r="A219" s="24" t="s">
         <v>1122</v>
       </c>
-      <c r="B219" s="20"/>
-      <c r="C219" s="20"/>
-      <c r="D219" s="20"/>
+      <c r="B219" s="24"/>
+      <c r="C219" s="24"/>
+      <c r="D219" s="24"/>
     </row>
     <row r="220" spans="1:5" ht="27.6">
       <c r="A220" s="5" t="s">
@@ -13298,12 +13480,12 @@
       </c>
     </row>
     <row r="223" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A223" s="20" t="s">
+      <c r="A223" s="24" t="s">
         <v>1125</v>
       </c>
-      <c r="B223" s="20"/>
-      <c r="C223" s="20"/>
-      <c r="D223" s="20"/>
+      <c r="B223" s="24"/>
+      <c r="C223" s="24"/>
+      <c r="D223" s="24"/>
     </row>
     <row r="224" spans="1:5">
       <c r="A224" s="5" t="s">
@@ -13334,12 +13516,12 @@
       </c>
     </row>
     <row r="227" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A227" s="20" t="s">
+      <c r="A227" s="24" t="s">
         <v>850</v>
       </c>
-      <c r="B227" s="20"/>
-      <c r="C227" s="20"/>
-      <c r="D227" s="20"/>
+      <c r="B227" s="24"/>
+      <c r="C227" s="24"/>
+      <c r="D227" s="24"/>
     </row>
     <row r="228" spans="1:4">
       <c r="A228" s="5" t="s">
@@ -13384,12 +13566,12 @@
       </c>
     </row>
     <row r="232" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A232" s="20" t="s">
+      <c r="A232" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B232" s="20"/>
-      <c r="C232" s="20"/>
-      <c r="D232" s="20"/>
+      <c r="B232" s="24"/>
+      <c r="C232" s="24"/>
+      <c r="D232" s="24"/>
     </row>
     <row r="233" spans="1:4" ht="55.2">
       <c r="A233" s="5" t="s">
@@ -13433,7 +13615,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="236" spans="1:4" ht="82.8">
+    <row r="236" spans="1:4" ht="96.6">
       <c r="A236" s="5" t="s">
         <v>1096</v>
       </c>
@@ -13448,12 +13630,12 @@
       </c>
     </row>
     <row r="238" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A238" s="20" t="s">
+      <c r="A238" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B238" s="20"/>
-      <c r="C238" s="20"/>
-      <c r="D238" s="20"/>
+      <c r="B238" s="24"/>
+      <c r="C238" s="24"/>
+      <c r="D238" s="24"/>
     </row>
     <row r="239" spans="1:4">
       <c r="A239" s="5" t="s">
@@ -13498,23 +13680,23 @@
       </c>
     </row>
     <row r="244" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A244" s="29" t="s">
+      <c r="A244" s="23" t="s">
         <v>1147</v>
       </c>
-      <c r="B244" s="29"/>
-      <c r="C244" s="29"/>
-      <c r="D244" s="29"/>
+      <c r="B244" s="23"/>
+      <c r="C244" s="23"/>
+      <c r="D244" s="23"/>
       <c r="E244" s="13" t="s">
         <v>1275</v>
       </c>
     </row>
     <row r="245" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A245" s="20" t="s">
+      <c r="A245" s="24" t="s">
         <v>1148</v>
       </c>
-      <c r="B245" s="20"/>
-      <c r="C245" s="20"/>
-      <c r="D245" s="20"/>
+      <c r="B245" s="24"/>
+      <c r="C245" s="24"/>
+      <c r="D245" s="24"/>
     </row>
     <row r="246" spans="1:5">
       <c r="A246" s="5" t="s">
@@ -13531,12 +13713,12 @@
       </c>
     </row>
     <row r="248" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A248" s="20" t="s">
+      <c r="A248" s="24" t="s">
         <v>1151</v>
       </c>
-      <c r="B248" s="20"/>
-      <c r="C248" s="20"/>
-      <c r="D248" s="20"/>
+      <c r="B248" s="24"/>
+      <c r="C248" s="24"/>
+      <c r="D248" s="24"/>
     </row>
     <row r="249" spans="1:5">
       <c r="A249" s="5" t="s">
@@ -13595,12 +13777,12 @@
       </c>
     </row>
     <row r="254" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A254" s="20" t="s">
+      <c r="A254" s="24" t="s">
         <v>1160</v>
       </c>
-      <c r="B254" s="20"/>
-      <c r="C254" s="20"/>
-      <c r="D254" s="20"/>
+      <c r="B254" s="24"/>
+      <c r="C254" s="24"/>
+      <c r="D254" s="24"/>
     </row>
     <row r="255" spans="1:5">
       <c r="A255" s="5" t="s">
@@ -13645,12 +13827,12 @@
       </c>
     </row>
     <row r="259" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A259" s="20" t="s">
+      <c r="A259" s="24" t="s">
         <v>1166</v>
       </c>
-      <c r="B259" s="20"/>
-      <c r="C259" s="20"/>
-      <c r="D259" s="20"/>
+      <c r="B259" s="24"/>
+      <c r="C259" s="24"/>
+      <c r="D259" s="24"/>
     </row>
     <row r="260" spans="1:4" ht="26.4">
       <c r="A260" s="5" t="s">
@@ -13681,12 +13863,12 @@
       </c>
     </row>
     <row r="263" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A263" s="20" t="s">
+      <c r="A263" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B263" s="20"/>
-      <c r="C263" s="20"/>
-      <c r="D263" s="20"/>
+      <c r="B263" s="24"/>
+      <c r="C263" s="24"/>
+      <c r="D263" s="24"/>
     </row>
     <row r="264" spans="1:4" ht="55.2">
       <c r="A264" s="5" t="s">
@@ -13745,12 +13927,12 @@
       </c>
     </row>
     <row r="269" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A269" s="20" t="s">
+      <c r="A269" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B269" s="20"/>
-      <c r="C269" s="20"/>
-      <c r="D269" s="20"/>
+      <c r="B269" s="24"/>
+      <c r="C269" s="24"/>
+      <c r="D269" s="24"/>
     </row>
     <row r="270" spans="1:4">
       <c r="A270" s="5" t="s">
@@ -13809,23 +13991,23 @@
       </c>
     </row>
     <row r="276" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A276" s="29" t="s">
+      <c r="A276" s="23" t="s">
         <v>1185</v>
       </c>
-      <c r="B276" s="29"/>
-      <c r="C276" s="29"/>
-      <c r="D276" s="29"/>
+      <c r="B276" s="23"/>
+      <c r="C276" s="23"/>
+      <c r="D276" s="23"/>
       <c r="E276" s="10" t="s">
         <v>1272</v>
       </c>
     </row>
     <row r="277" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A277" s="20" t="s">
+      <c r="A277" s="24" t="s">
         <v>1186</v>
       </c>
-      <c r="B277" s="20"/>
-      <c r="C277" s="20"/>
-      <c r="D277" s="20"/>
+      <c r="B277" s="24"/>
+      <c r="C277" s="24"/>
+      <c r="D277" s="24"/>
     </row>
     <row r="278" spans="1:5" ht="41.4">
       <c r="A278" s="5" t="s">
@@ -13898,12 +14080,12 @@
       </c>
     </row>
     <row r="284" spans="1:5" ht="19.95" customHeight="1">
-      <c r="A284" s="20" t="s">
+      <c r="A284" s="24" t="s">
         <v>1196</v>
       </c>
-      <c r="B284" s="20"/>
-      <c r="C284" s="20"/>
-      <c r="D284" s="20"/>
+      <c r="B284" s="24"/>
+      <c r="C284" s="24"/>
+      <c r="D284" s="24"/>
     </row>
     <row r="285" spans="1:5">
       <c r="A285" s="5" t="s">
@@ -14032,12 +14214,12 @@
       </c>
     </row>
     <row r="295" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A295" s="20" t="s">
+      <c r="A295" s="24" t="s">
         <v>1214</v>
       </c>
-      <c r="B295" s="20"/>
-      <c r="C295" s="20"/>
-      <c r="D295" s="20"/>
+      <c r="B295" s="24"/>
+      <c r="C295" s="24"/>
+      <c r="D295" s="24"/>
     </row>
     <row r="296" spans="1:4">
       <c r="A296" s="5" t="s">
@@ -14082,12 +14264,12 @@
       </c>
     </row>
     <row r="300" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A300" s="20" t="s">
+      <c r="A300" s="24" t="s">
         <v>1221</v>
       </c>
-      <c r="B300" s="20"/>
-      <c r="C300" s="20"/>
-      <c r="D300" s="20"/>
+      <c r="B300" s="24"/>
+      <c r="C300" s="24"/>
+      <c r="D300" s="24"/>
     </row>
     <row r="301" spans="1:4" ht="39.6">
       <c r="A301" s="5" t="s">
@@ -14146,12 +14328,12 @@
       </c>
     </row>
     <row r="306" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A306" s="20" t="s">
+      <c r="A306" s="24" t="s">
         <v>1229</v>
       </c>
-      <c r="B306" s="20"/>
-      <c r="C306" s="20"/>
-      <c r="D306" s="20"/>
+      <c r="B306" s="24"/>
+      <c r="C306" s="24"/>
+      <c r="D306" s="24"/>
     </row>
     <row r="307" spans="1:4">
       <c r="A307" s="5" t="s">
@@ -14294,12 +14476,12 @@
       </c>
     </row>
     <row r="318" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A318" s="20" t="s">
+      <c r="A318" s="24" t="s">
         <v>1248</v>
       </c>
-      <c r="B318" s="20"/>
-      <c r="C318" s="20"/>
-      <c r="D318" s="20"/>
+      <c r="B318" s="24"/>
+      <c r="C318" s="24"/>
+      <c r="D318" s="24"/>
     </row>
     <row r="319" spans="1:4" ht="27.6">
       <c r="A319" s="5" t="s">
@@ -14344,12 +14526,12 @@
       </c>
     </row>
     <row r="323" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A323" s="20" t="s">
+      <c r="A323" s="24" t="s">
         <v>862</v>
       </c>
-      <c r="B323" s="20"/>
-      <c r="C323" s="20"/>
-      <c r="D323" s="20"/>
+      <c r="B323" s="24"/>
+      <c r="C323" s="24"/>
+      <c r="D323" s="24"/>
     </row>
     <row r="324" spans="1:4">
       <c r="A324" s="5" t="s">
@@ -14394,12 +14576,12 @@
       </c>
     </row>
     <row r="328" spans="1:4" ht="19.95" customHeight="1">
-      <c r="A328" s="20" t="s">
+      <c r="A328" s="24" t="s">
         <v>855</v>
       </c>
-      <c r="B328" s="20"/>
-      <c r="C328" s="20"/>
-      <c r="D328" s="20"/>
+      <c r="B328" s="24"/>
+      <c r="C328" s="24"/>
+      <c r="D328" s="24"/>
     </row>
     <row r="329" spans="1:4" ht="96.6">
       <c r="A329" s="5" t="s">
@@ -14555,22 +14737,22 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:5" ht="18">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="39" t="s">
         <v>1278</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="41" t="s">
         <v>1279</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="14" t="s">
@@ -14637,13 +14819,13 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="41" t="s">
         <v>1290</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="40"/>
+      <c r="E10" s="40"/>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="14" t="s">
@@ -14652,11 +14834,11 @@
       <c r="B11" s="14" t="s">
         <v>1291</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="35"/>
-      <c r="E11" s="36"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44"/>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="15">
@@ -14705,186 +14887,238 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AFF2AF-D4BC-4BC0-A7E1-D98D2CA71943}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="6.88671875" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="49.88671875" customWidth="1"/>
     <col min="3" max="3" width="90.88671875" customWidth="1"/>
     <col min="4" max="4" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="21" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+    </row>
+    <row r="3" spans="1:4" ht="15.6">
+      <c r="A3" s="23" t="s">
         <v>1298</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-    </row>
-    <row r="3" spans="1:4" ht="15.6">
-      <c r="A3" s="29" t="s">
-        <v>1299</v>
-      </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-    </row>
-    <row r="5" spans="1:4" ht="138">
-      <c r="A5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>831</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>832</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="82.8">
-      <c r="A6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>833</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>834</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="110.4">
-      <c r="A7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>835</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>836</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="165.6">
-      <c r="A8" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>837</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>838</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>26</v>
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+    </row>
+    <row r="5" spans="1:4" ht="15" thickBot="1">
+      <c r="B5" s="17" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" thickBot="1">
+      <c r="A6" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>1304</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>1305</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1">
+      <c r="B7" s="18" t="s">
+        <v>1306</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>1307</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="B8" s="18" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1309</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1324</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="B9" s="18" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>1311</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1323</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="20" t="s">
-        <v>839</v>
-      </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-    </row>
-    <row r="11" spans="1:4" ht="124.2">
-      <c r="A11" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>840</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>841</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="409.2">
-      <c r="A12" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>842</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>843</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="151.80000000000001">
-      <c r="A13" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>844</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>845</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="82.8">
-      <c r="A14" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>846</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>847</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="220.8">
-      <c r="A15" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>848</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>849</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="20" t="s">
-        <v>850</v>
-      </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="B10" s="18" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="B11" s="18" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>1322</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="B12" s="18" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>1325</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="B13" s="18" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="B14" s="20" t="s">
+        <v>1314</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>1315</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="B15" s="20" t="s">
+        <v>1316</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>1317</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="C16" s="18" t="s">
+        <v>1318</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="C17" s="18" t="s">
+        <v>1319</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="C19" s="18" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4">
+      <c r="B21" s="45" t="s">
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4">
+      <c r="B22" s="12"/>
+    </row>
+    <row r="23" spans="2:4">
+      <c r="B23" s="12" t="s">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="B24" s="12" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4">
+      <c r="B25" s="12" t="s">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4">
+      <c r="B26" s="12" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4">
+      <c r="B27" s="12" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4">
+      <c r="B28" s="12" t="s">
+        <v>1337</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4">
+      <c r="B29" s="18" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4">
+      <c r="B30" s="18"/>
+    </row>
+    <row r="31" spans="2:4">
+      <c r="B31" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>